<commit_message>
feat: add mandatory reward choice
</commit_message>
<xml_diff>
--- a/data/爱乐之城-表演道具验证配置.xlsx
+++ b/data/爱乐之城-表演道具验证配置.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="Rdbdf126a8384426a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规则配置" sheetId="2" r:id="R10dcc62b2e7c4e90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品质配置" sheetId="3" r:id="R0de5a2f93aeb464c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表演规则" sheetId="4" r:id="R71d6d9e2d95c4c0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发挥档位" sheetId="5" r:id="Rf9100aaf53814b4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="现场事件" sheetId="6" r:id="Rdd850c5358ae4d7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="种类表演特性" sheetId="7" r:id="R9b63ef871e9e400c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="道具配置" sheetId="8" r:id="R5b6c2283fec64bd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R846b802dde344b4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规则配置" sheetId="2" r:id="Rbe3914927f57488b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品质配置" sheetId="3" r:id="Reaf9333dd3174a09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表演规则" sheetId="4" r:id="Radc0acf2d4664340"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发挥档位" sheetId="5" r:id="R1ba889e2f08947d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="现场事件" sheetId="6" r:id="Rb80dd382fca14ca4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="种类表演特性" sheetId="7" r:id="R77a04a17b1b64e7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="道具配置" sheetId="8" r:id="R654f16db06414ce1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -274,7 +274,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ValidatorRulesTable" displayName="ValidatorRulesTable" ref="A1:D15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ValidatorRulesTable" displayName="ValidatorRulesTable" ref="A1:D16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="键名"/>
     <x:tableColumn id="2" name="值"/>
@@ -611,7 +611,7 @@
         <x:v>试玩成长</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>初始随机获得1件紫色与1件蓝色道具；默认每完成3次表演，从尚未解锁的道具中随机解锁新道具。</x:v>
+        <x:v>初始随机获得1件紫色与1件蓝色道具；默认每完成3次表演，随机展示3件尚未解锁的道具，玩家选择1件获得。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
@@ -619,7 +619,7 @@
         <x:v>规则配置</x:v>
       </x:c>
       <x:c r="B6" s="13" t="str">
-        <x:v>修改格子、体力、扩格节奏、试玩初始道具与单场解锁数量等参数。键名不要修改。</x:v>
+        <x:v>修改格子、体力、扩格节奏、试玩初始道具、奖励候选数量与单次获得数量等参数。键名不要修改。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="38" customHeight="1">
@@ -930,10 +930,24 @@
         <x:v>本机最多保留的表演日志条数</x:v>
       </x:c>
     </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>trial_reward_choice_count</x:v>
+      </x:c>
+      <x:c r="B16" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>整数</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>试玩模式每次奖励随机展示的候选道具数量</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c0ec66da7054a9e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2721456420b4b1e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1037,7 +1051,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2933d5363b6245f7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc3e9332a1314be0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1245,7 +1259,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbeb65e883a7f447a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64d88c0edc6442a8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1365,7 +1379,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5016e42cc93a4d09"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d8c9dd245f249a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1607,7 +1621,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5becb30bc16f49f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9b8297729164d1e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1745,7 +1759,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6d7701dd8744339"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83c82435d9464d53"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6550,7 +6564,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24131ed77ca64e9f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6563558ebca4d1a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Revise prop effects and reward choices
</commit_message>
<xml_diff>
--- a/data/爱乐之城-表演道具验证配置.xlsx
+++ b/data/爱乐之城-表演道具验证配置.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R846b802dde344b4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规则配置" sheetId="2" r:id="Rbe3914927f57488b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品质配置" sheetId="3" r:id="Reaf9333dd3174a09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表演规则" sheetId="4" r:id="Radc0acf2d4664340"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发挥档位" sheetId="5" r:id="R1ba889e2f08947d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="现场事件" sheetId="6" r:id="Rb80dd382fca14ca4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="种类表演特性" sheetId="7" r:id="R77a04a17b1b64e7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="道具配置" sheetId="8" r:id="R654f16db06414ce1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="Rd97b1f70421d45c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规则配置" sheetId="2" r:id="Rd81a7ed8725f4157"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品质配置" sheetId="3" r:id="R75fc9848daab41e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表演规则" sheetId="4" r:id="R5f1b896861f947d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发挥档位" sheetId="5" r:id="R3526c4e186b24d73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="现场事件" sheetId="6" r:id="R74a43003582a4165"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="种类表演特性" sheetId="7" r:id="R7b660783b5b54f54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="道具配置" sheetId="8" r:id="R6f862d8f5aa24bc1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -274,7 +274,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ValidatorRulesTable" displayName="ValidatorRulesTable" ref="A1:D16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ValidatorRulesTable" displayName="ValidatorRulesTable" ref="A1:D18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="键名"/>
     <x:tableColumn id="2" name="值"/>
@@ -368,11 +368,11 @@
     <x:tableColumn id="11" name="限制范围"/>
     <x:tableColumn id="12" name="限制键"/>
     <x:tableColumn id="13" name="限制数量"/>
-    <x:tableColumn id="14" name="基础人气Lv1"/>
-    <x:tableColumn id="15" name="基础人气Lv2"/>
-    <x:tableColumn id="16" name="基础人气Lv3"/>
-    <x:tableColumn id="17" name="基础人气Lv4"/>
-    <x:tableColumn id="18" name="基础人气Lv5"/>
+    <x:tableColumn id="14" name="基础表演值Lv1"/>
+    <x:tableColumn id="15" name="基础表演值Lv2"/>
+    <x:tableColumn id="16" name="基础表演值Lv3"/>
+    <x:tableColumn id="17" name="基础表演值Lv4"/>
+    <x:tableColumn id="18" name="基础表演值Lv5"/>
     <x:tableColumn id="19" name="效果值Lv1"/>
     <x:tableColumn id="20" name="效果值Lv2"/>
     <x:tableColumn id="21" name="效果值Lv3"/>
@@ -611,7 +611,7 @@
         <x:v>试玩成长</x:v>
       </x:c>
       <x:c r="B5" s="13" t="str">
-        <x:v>初始随机获得1件紫色与1件蓝色道具；默认每完成3次表演，随机展示3件尚未解锁的道具，玩家选择1件获得。</x:v>
+        <x:v>初始随机获得1件紫色与1件蓝色道具；每完成3次表演进入三选一，50%概率首个选项为解锁背包格。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
@@ -619,7 +619,7 @@
         <x:v>规则配置</x:v>
       </x:c>
       <x:c r="B6" s="13" t="str">
-        <x:v>修改格子、体力、扩格节奏、试玩初始道具、奖励候选数量与单次获得数量等参数。键名不要修改。</x:v>
+        <x:v>修改背包、体力、奖励频率、选格概率、单次选格数量与试玩初始道具等参数。键名不要修改。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="38" customHeight="1">
@@ -659,7 +659,7 @@
         <x:v>种类表演特性</x:v>
       </x:c>
       <x:c r="B11" s="13" t="str">
-        <x:v>配置六类道具被聚光选中的权重，以及节拍判定窗口修正。</x:v>
+        <x:v>内部配置六类道具被聚光选中的权重，以及节拍判定窗口修正；种类不在玩家界面展示。</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="38" customHeight="1">
@@ -667,7 +667,7 @@
         <x:v>道具配置</x:v>
       </x:c>
       <x:c r="B12" s="13" t="str">
-        <x:v>60 件道具的名称、分类、形状、限制、五级数值、效果规则与文案。</x:v>
+        <x:v>60 件道具的名称、内部种类、标签、形状、限制、五级数值、效果规则与文案。效果条件只使用标签。</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="38" customHeight="1">
@@ -683,7 +683,7 @@
         <x:v>五级数值</x:v>
       </x:c>
       <x:c r="B14" s="13" t="str">
-        <x:v>基础人气与效果值分别配置 Lv.1—Lv.5。等级不改变形状、限制和触发条件。</x:v>
+        <x:v>基础表演值与效果值分别配置 Lv.1—Lv.5。百分比效果以整数填写，例如8代表8%。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="38" customHeight="1">
@@ -792,7 +792,7 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="19" t="str">
-        <x:v>performances_per_expand</x:v>
+        <x:v>stamina_per_performance</x:v>
       </x:c>
       <x:c r="B6" s="25" t="n">
         <x:v>3</x:v>
@@ -801,54 +801,54 @@
         <x:v>整数</x:v>
       </x:c>
       <x:c r="D6" s="21" t="str">
-        <x:v>每完成多少次表演获得 1 次扩格</x:v>
+        <x:v>每次表演消耗体力</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="19" t="str">
-        <x:v>stamina_per_performance</x:v>
+        <x:v>initial_item_level</x:v>
       </x:c>
       <x:c r="B7" s="25" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C7" s="20" t="str">
         <x:v>整数</x:v>
       </x:c>
       <x:c r="D7" s="21" t="str">
-        <x:v>每次表演消耗体力</x:v>
+        <x:v>仓库初始道具等级</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="19" t="str">
-        <x:v>initial_item_level</x:v>
+        <x:v>max_item_level</x:v>
       </x:c>
       <x:c r="B8" s="25" t="n">
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C8" s="20" t="str">
         <x:v>整数</x:v>
       </x:c>
       <x:c r="D8" s="21" t="str">
-        <x:v>仓库初始道具等级</x:v>
+        <x:v>测试器允许的最高等级</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="19" t="str">
-        <x:v>max_item_level</x:v>
+        <x:v>test_initial_copies_each</x:v>
       </x:c>
       <x:c r="B9" s="25" t="n">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C9" s="20" t="str">
         <x:v>整数</x:v>
       </x:c>
       <x:c r="D9" s="21" t="str">
-        <x:v>测试器允许的最高等级</x:v>
+        <x:v>测试模式初始拥有每种道具的件数</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="19" t="str">
-        <x:v>test_initial_copies_each</x:v>
+        <x:v>trial_initial_purple_count</x:v>
       </x:c>
       <x:c r="B10" s="25" t="n">
         <x:v>1</x:v>
@@ -857,12 +857,12 @@
         <x:v>整数</x:v>
       </x:c>
       <x:c r="D10" s="21" t="str">
-        <x:v>测试模式初始拥有每种道具的件数</x:v>
+        <x:v>试玩模式初始紫色道具数量</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="19" t="str">
-        <x:v>trial_initial_purple_count</x:v>
+        <x:v>trial_initial_blue_count</x:v>
       </x:c>
       <x:c r="B11" s="25" t="n">
         <x:v>1</x:v>
@@ -871,83 +871,111 @@
         <x:v>整数</x:v>
       </x:c>
       <x:c r="D11" s="21" t="str">
-        <x:v>试玩模式初始紫色道具数量</x:v>
+        <x:v>试玩模式初始蓝色道具数量</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="19" t="str">
-        <x:v>trial_initial_blue_count</x:v>
+        <x:v>trial_performances_per_reward</x:v>
       </x:c>
       <x:c r="B12" s="25" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C12" s="20" t="str">
         <x:v>整数</x:v>
       </x:c>
       <x:c r="D12" s="21" t="str">
-        <x:v>试玩模式初始蓝色道具数量</x:v>
+        <x:v>试玩模式每完成多少次表演解锁一批新道具</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="19" t="str">
-        <x:v>trial_performances_per_reward</x:v>
+        <x:v>trial_rewards_per_performance</x:v>
       </x:c>
       <x:c r="B13" s="25" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C13" s="20" t="str">
         <x:v>整数</x:v>
       </x:c>
       <x:c r="D13" s="21" t="str">
-        <x:v>试玩模式每完成多少次表演解锁一批新道具</x:v>
+        <x:v>试玩模式每次解锁的新道具数量</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="19" t="str">
-        <x:v>trial_rewards_per_performance</x:v>
+        <x:v>trial_reward_choice_count</x:v>
       </x:c>
       <x:c r="B14" s="25" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C14" s="20" t="str">
         <x:v>整数</x:v>
       </x:c>
       <x:c r="D14" s="21" t="str">
-        <x:v>试玩模式每次解锁的新道具数量</x:v>
+        <x:v>试玩模式每次奖励展示的候选数量</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="22" t="str">
+      <x:c r="A15" s="19" t="str">
+        <x:v>reward_unlock_option_chance</x:v>
+      </x:c>
+      <x:c r="B15" s="25" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C15" s="20" t="str">
+        <x:v>小数</x:v>
+      </x:c>
+      <x:c r="D15" s="21" t="str">
+        <x:v>每次三选一的首项为解锁格子的概率</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="19" t="str">
+        <x:v>reward_unlock_count</x:v>
+      </x:c>
+      <x:c r="B16" s="25" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C16" s="20" t="str">
+        <x:v>整数</x:v>
+      </x:c>
+      <x:c r="D16" s="21" t="str">
+        <x:v>普通奖励轮选择格子时获得的扩格次数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="19" t="str">
+        <x:v>reward_highest_quality_unlock_count</x:v>
+      </x:c>
+      <x:c r="B17" s="25" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C17" s="20" t="str">
+        <x:v>整数</x:v>
+      </x:c>
+      <x:c r="D17" s="21" t="str">
+        <x:v>候选含最高品质道具时选择格子获得的扩格次数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="22" t="str">
         <x:v>max_log_entries</x:v>
       </x:c>
-      <x:c r="B15" s="26" t="n">
+      <x:c r="B18" s="26" t="n">
         <x:v>500</x:v>
       </x:c>
-      <x:c r="C15" s="23" t="str">
+      <x:c r="C18" s="23" t="str">
         <x:v>整数</x:v>
       </x:c>
-      <x:c r="D15" s="24" t="str">
+      <x:c r="D18" s="24" t="str">
         <x:v>本机最多保留的表演日志条数</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" t="str">
-        <x:v>trial_reward_choice_count</x:v>
-      </x:c>
-      <x:c r="B16" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C16" t="str">
-        <x:v>整数</x:v>
-      </x:c>
-      <x:c r="D16" t="str">
-        <x:v>试玩模式每次奖励随机展示的候选道具数量</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2721456420b4b1e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e14deed53be46d5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1051,7 +1079,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc3e9332a1314be0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re69cb55fc2324f5c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1259,7 +1287,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64d88c0edc6442a8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra19878cdde9143c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1379,7 +1407,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d8c9dd245f249a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1536f8f27aa4162"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1621,7 +1649,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9b8297729164d1e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R707dd46217fc488f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1759,7 +1787,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83c82435d9464d53"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R300ff96c92c34fe8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1781,11 +1809,11 @@
     <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="16" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="16" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="10.380000114440918" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="10.380000114440918" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="10.380000114440918" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="10.380000114440918" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="10.380000114440918" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="12.25" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="12.25" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="12.25" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="12.25" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="12.25" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="8.5" hidden="0" customWidth="1"/>
     <x:col min="20" max="20" width="8.5" hidden="0" customWidth="1"/>
     <x:col min="21" max="21" width="8.5" hidden="0" customWidth="1"/>
@@ -1836,19 +1864,19 @@
         <x:v>限制数量</x:v>
       </x:c>
       <x:c r="N1" s="17" t="str">
-        <x:v>基础人气Lv1</x:v>
+        <x:v>基础表演值Lv1</x:v>
       </x:c>
       <x:c r="O1" s="17" t="str">
-        <x:v>基础人气Lv2</x:v>
+        <x:v>基础表演值Lv2</x:v>
       </x:c>
       <x:c r="P1" s="17" t="str">
-        <x:v>基础人气Lv3</x:v>
+        <x:v>基础表演值Lv3</x:v>
       </x:c>
       <x:c r="Q1" s="17" t="str">
-        <x:v>基础人气Lv4</x:v>
+        <x:v>基础表演值Lv4</x:v>
       </x:c>
       <x:c r="R1" s="17" t="str">
-        <x:v>基础人气Lv5</x:v>
+        <x:v>基础表演值Lv5</x:v>
       </x:c>
       <x:c r="S1" s="17" t="str">
         <x:v>效果值Lv1</x:v>
@@ -1929,25 +1957,25 @@
         <x:v>308</x:v>
       </x:c>
       <x:c r="S2" s="43" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="T2" s="43" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="U2" s="43" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="V2" s="43" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="W2" s="43" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="T2" s="43" t="n">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="U2" s="43" t="n">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="V2" s="43" t="n">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="W2" s="43" t="n">
-        <x:v>73</x:v>
-      </x:c>
       <x:c r="X2" s="40" t="str">
-        <x:v>{"type":"count","scope":"global","filter":{"category":["弦乐器","管乐器","打击乐器"]},"cap":6,"excludeSource":true,"excludeAdjacent":false,"directions":[],"recipient":"self"}</x:v>
+        <x:v>{"type":"condition","clauses":[{"scope":"global","filter":{"tag1":["提琴声部"]},"min":1,"max":null,"cap":null,"excludeSource":true,"directions":[]},{"scope":"global","filter":{"tag1":["木管声部"]},"min":1,"max":null,"cap":null,"excludeSource":true,"directions":[]},{"scope":"global","filter":{"tag1":["管弦打击"]},"min":1,"max":null,"cap":null,"excludeSource":true,"directions":[]}],"valueMode":"percent","recipient":"self"}</x:v>
       </x:c>
       <x:c r="Y2" s="44" t="str">
-        <x:v>背包中每有1件弦乐器、管乐器或打击乐器，自身增加[30／37／45／52／73]人气；合计最多6件，不计自身</x:v>
+        <x:v>背包中提琴声部、木管声部和管弦打击各至少1件时，自身表演值增加[12／15／19／24／30]%</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
@@ -2007,25 +2035,25 @@
         <x:v>208</x:v>
       </x:c>
       <x:c r="S3" s="43" t="n">
-        <x:v>24</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="T3" s="43" t="n">
-        <x:v>31</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="U3" s="43" t="n">
-        <x:v>40</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="V3" s="43" t="n">
-        <x:v>49</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="W3" s="43" t="n">
-        <x:v>60</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="X3" s="40" t="str">
-        <x:v>{"type":"count","scope":"adjacent","filter":{"category":["键盘乐器","弦乐器","管乐器","打击乐器"],"tag2":["古典"]},"cap":4,"excludeSource":true,"excludeAdjacent":false,"directions":[],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["古典"]},"cap":4,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y3" s="44" t="str">
-        <x:v>每相邻1件古典乐器，自身增加[24／31／40／49／60]人气，最多4件</x:v>
+        <x:v>使相邻的古典乐器标签道具各增加[5／6／8／10／12]%表演值，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
@@ -2085,25 +2113,25 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="S4" s="43" t="n">
-        <x:v>62</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="T4" s="43" t="n">
-        <x:v>81</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="U4" s="43" t="n">
-        <x:v>102</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="V4" s="43" t="n">
-        <x:v>127</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="W4" s="43" t="n">
-        <x:v>155</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="X4" s="40" t="str">
-        <x:v>{"type":"condition","clauses":[{"scope":"direction","filter":{"category":["弦乐器"]},"min":1,"max":null,"cap":1,"excludeSource":true,"directions":["left"]},{"scope":"direction","filter":{"category":["管乐器"]},"min":1,"max":null,"cap":1,"excludeSource":true,"directions":["right"]}],"recipient":"self"}</x:v>
+        <x:v>{"type":"groupBuff","clauses":[{"scope":"direction","filter":{"tag1":["提琴声部","拨弦声部"]},"min":1,"max":null,"cap":null,"excludeSource":true,"directions":["left"]},{"scope":"direction","filter":{"tag1":["木管声部","铜管声部"]},"min":1,"max":null,"cap":null,"excludeSource":true,"directions":["right"]}],"recipients":{"scope":"direction","directions":["left","right"],"filter":{"tag1":["提琴声部","拨弦声部","木管声部","铜管声部"]},"cap":4,"includeSource":false},"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y4" s="44" t="str">
-        <x:v>左侧至少有1件弦乐器且右侧至少有1件管乐器时，自身增加[62／81／102／127／155]人气；两侧各检查最多1件</x:v>
+        <x:v>左侧至少有1件提琴声部或拨弦声部，且右侧至少有1件木管声部或铜管声部时，使两侧符合条件的道具各增加[5／6／8／10／12]%表演值，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="42" customHeight="1">
@@ -2163,25 +2191,25 @@
         <x:v>123</x:v>
       </x:c>
       <x:c r="S5" s="43" t="n">
-        <x:v>13</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="T5" s="43" t="n">
-        <x:v>17</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="U5" s="43" t="n">
-        <x:v>21</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="V5" s="43" t="n">
-        <x:v>27</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="W5" s="43" t="n">
-        <x:v>33</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="X5" s="40" t="str">
-        <x:v>{"type":"count","scope":"direction","filter":{"any":true},"cap":4,"excludeSource":true,"excludeAdjacent":false,"directions":["up","down"],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"]},"cap":4,"excludeSource":true,"directions":["up","down"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y5" s="44" t="str">
-        <x:v>上方与下方每有1件道具，自身增加[13／17／21／27／33]人气，两个方向合计最多4件</x:v>
+        <x:v>使上方和下方的乐器标签道具各增加[5／7／9／11／14]表演值，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
@@ -2241,25 +2269,25 @@
         <x:v>123</x:v>
       </x:c>
       <x:c r="S6" s="43" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="T6" s="43" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="U6" s="43" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="V6" s="43" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="W6" s="43" t="n">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="T6" s="43" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="U6" s="43" t="n">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="V6" s="43" t="n">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="W6" s="43" t="n">
-        <x:v>35</x:v>
-      </x:c>
       <x:c r="X6" s="40" t="str">
-        <x:v>{"type":"count","scope":"global","filter":{"category":["管乐器"],"tag2":["现代"]},"cap":4,"excludeSource":true,"excludeAdjacent":false,"directions":[],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"global","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["现代"]},"cap":4,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y6" s="44" t="str">
-        <x:v>背包中每有1件现代管乐器，自身增加[14／18／23／29／35]人气，最多4件，不计自身</x:v>
+        <x:v>使背包中的现代乐器标签道具各增加[5／7／9／11／14]表演值，最多4件，不计自身</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
@@ -2319,25 +2347,25 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="S7" s="43" t="n">
-        <x:v>44</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="T7" s="43" t="n">
-        <x:v>57</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="U7" s="43" t="n">
-        <x:v>73</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="V7" s="43" t="n">
-        <x:v>90</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="W7" s="43" t="n">
-        <x:v>110</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="X7" s="40" t="str">
-        <x:v>{"type":"condition","clauses":[{"scope":"adjacent","filter":{"any":true},"min":null,"max":2,"cap":null,"excludeSource":true,"directions":[]}],"recipient":"self"}</x:v>
+        <x:v>{"type":"condition","clauses":[{"scope":"adjacent","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"]},"min":null,"max":2,"cap":null,"excludeSource":true,"directions":[]}],"valueMode":"absolute","recipient":"self"}</x:v>
       </x:c>
       <x:c r="Y7" s="44" t="str">
-        <x:v>相邻道具不超过2件时，自身增加[44／57／73／90／110]人气；相邻数量只检查一次</x:v>
+        <x:v>相邻的乐器标签道具不超过2件时，自身增加[38／49／63／78／95]表演值</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
@@ -2397,25 +2425,25 @@
         <x:v>73</x:v>
       </x:c>
       <x:c r="S8" s="43" t="n">
-        <x:v>13</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="T8" s="43" t="n">
-        <x:v>17</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="U8" s="43" t="n">
-        <x:v>21</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="V8" s="43" t="n">
-        <x:v>27</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="W8" s="43" t="n">
-        <x:v>33</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="X8" s="40" t="str">
-        <x:v>{"type":"count","scope":"adjacent","filter":{"any":true},"cap":2,"excludeSource":true,"excludeAdjacent":false,"directions":[],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y8" s="44" t="str">
-        <x:v>每相邻1件道具，自身增加[13／17／21／27／33]人气，最多2件</x:v>
+        <x:v>使相邻的乐器标签道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
@@ -2475,25 +2503,25 @@
         <x:v>73</x:v>
       </x:c>
       <x:c r="S9" s="43" t="n">
-        <x:v>14</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="T9" s="43" t="n">
-        <x:v>18</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="U9" s="43" t="n">
-        <x:v>23</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="V9" s="43" t="n">
-        <x:v>29</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="W9" s="43" t="n">
-        <x:v>35</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="X9" s="40" t="str">
-        <x:v>{"type":"count","scope":"direction","filter":{"any":true},"cap":2,"excludeSource":true,"excludeAdjacent":false,"directions":["left"],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"]},"cap":2,"excludeSource":true,"directions":["left"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y9" s="44" t="str">
-        <x:v>左侧每有1件道具，自身增加[14／18／23／29／35]人气，最多2件</x:v>
+        <x:v>使左侧的乐器标签道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
@@ -2553,25 +2581,25 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="S10" s="43" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="T10" s="43" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="U10" s="43" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="V10" s="43" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="T10" s="43" t="n">
+      <x:c r="W10" s="43" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="U10" s="43" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="V10" s="43" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="W10" s="43" t="n">
-        <x:v>20</x:v>
-      </x:c>
       <x:c r="X10" s="40" t="str">
-        <x:v>{"type":"count","scope":"global","filter":{"minArea":4},"cap":3,"excludeSource":true,"excludeAdjacent":false,"directions":[],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"global","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"minArea":4},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y10" s="44" t="str">
-        <x:v>背包中每有1件占用4格及以上的道具，自身增加[8／10／13／16／20]人气，最多3件，不计自身</x:v>
+        <x:v>使背包中占用4格及以上的乐器标签道具各增加[4／5／6／8／10]表演值，最多3件，不计自身</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
@@ -2631,25 +2659,25 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="S11" s="43" t="n">
-        <x:v>11</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="T11" s="43" t="n">
-        <x:v>14</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="U11" s="43" t="n">
-        <x:v>18</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="V11" s="43" t="n">
-        <x:v>23</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="W11" s="43" t="n">
-        <x:v>28</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="X11" s="40" t="str">
-        <x:v>{"type":"count","scope":"direction","filter":{"any":true},"cap":2,"excludeSource":true,"excludeAdjacent":false,"directions":["right"],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"]},"cap":2,"excludeSource":true,"directions":["right"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y11" s="44" t="str">
-        <x:v>右侧每有1件道具，自身增加[11／14／18／23／28]人气，最多2件</x:v>
+        <x:v>使右侧的乐器标签道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
@@ -2709,25 +2737,25 @@
         <x:v>255</x:v>
       </x:c>
       <x:c r="S12" s="43" t="n">
-        <x:v>24</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="T12" s="43" t="n">
-        <x:v>29</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="U12" s="43" t="n">
-        <x:v>35</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="V12" s="43" t="n">
-        <x:v>42</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="W12" s="43" t="n">
-        <x:v>60</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="X12" s="40" t="str">
-        <x:v>{"type":"count","scope":"global","filter":{"tag1":["提琴声部"]},"cap":6,"excludeSource":true,"excludeAdjacent":false,"directions":[],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"global","filter":{"tag1":["提琴声部"]},"cap":6,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y12" s="44" t="str">
-        <x:v>背包中每有1件提琴声部道具，自身增加[24／29／35／42／60]人气，最多6件，不计自身</x:v>
+        <x:v>使背包中的提琴声部道具各增加[3／4／5／6／8]%表演值，最多6件</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
@@ -2787,25 +2815,25 @@
         <x:v>158</x:v>
       </x:c>
       <x:c r="S13" s="43" t="n">
-        <x:v>14</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="T13" s="43" t="n">
-        <x:v>18</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="U13" s="43" t="n">
-        <x:v>23</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="V13" s="43" t="n">
-        <x:v>29</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="W13" s="43" t="n">
-        <x:v>35</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="X13" s="40" t="str">
-        <x:v>{"type":"count","scope":"global","filter":{"tag1":["提琴声部"]},"cap":5,"excludeSource":true,"excludeAdjacent":false,"directions":[],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"global","filter":{"tag1":["提琴声部"]},"cap":5,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y13" s="44" t="str">
-        <x:v>背包中每有1件其他提琴声部道具，自身增加[14／18／23／29／35]人气，最多5件，不计自身</x:v>
+        <x:v>使背包中的其他提琴声部道具各增加[3／4／5／6／8]%表演值，最多5件</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
@@ -2865,25 +2893,25 @@
         <x:v>158</x:v>
       </x:c>
       <x:c r="S14" s="43" t="n">
-        <x:v>19</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="T14" s="43" t="n">
-        <x:v>25</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="U14" s="43" t="n">
-        <x:v>31</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="V14" s="43" t="n">
-        <x:v>39</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="W14" s="43" t="n">
-        <x:v>48</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="X14" s="40" t="str">
-        <x:v>{"type":"count","scope":"global","filter":{"tag1":["提琴声部"]},"cap":4,"excludeSource":true,"excludeAdjacent":true,"directions":[],"recipient":"self"}</x:v>
+        <x:v>{"type":"count","scope":"global","filter":{"tag1":["提琴声部"]},"cap":4,"excludeSource":true,"excludeAdjacent":true,"directions":[],"valueMode":"percent","recipient":"self"}</x:v>
       </x:c>
       <x:c r="Y14" s="44" t="str">
-        <x:v>背包中每有1件与自身不相邻的提琴声部道具，自身增加[19／25／31／39／48]人气，最多4件，不计自身</x:v>
+        <x:v>背包中每有1件与自身不相邻的提琴声部道具，自身表演值增加[2／3／4／5／6]%，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
@@ -2943,25 +2971,25 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S15" s="43" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="T15" s="43" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="U15" s="43" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="T15" s="43" t="n">
+      <x:c r="V15" s="43" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="U15" s="43" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="V15" s="43" t="n">
-        <x:v>14</x:v>
-      </x:c>
       <x:c r="W15" s="43" t="n">
-        <x:v>18</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="X15" s="40" t="str">
-        <x:v>{"type":"count","scope":"adjacent","filter":{"name":["音乐会小提琴"]},"cap":3,"excludeSource":true,"excludeAdjacent":false,"directions":[],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["提琴声部"]},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y15" s="44" t="str">
-        <x:v>每相邻1件其他音乐会小提琴，自身增加[7／9／12／14／18]人气，最多3件</x:v>
+        <x:v>使相邻的其他提琴声部道具各增加[4／5／7／9／11]表演值，最多3件</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
@@ -3021,25 +3049,25 @@
         <x:v>75</x:v>
       </x:c>
       <x:c r="S16" s="43" t="n">
-        <x:v>10</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="T16" s="43" t="n">
-        <x:v>13</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="U16" s="43" t="n">
-        <x:v>17</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="V16" s="43" t="n">
-        <x:v>21</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="W16" s="43" t="n">
-        <x:v>25</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="X16" s="40" t="str">
-        <x:v>{"type":"count","scope":"adjacent","filter":{"tag1":["提琴声部"]},"cap":3,"excludeSource":true,"excludeAdjacent":false,"directions":[],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["提琴声部"]},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y16" s="44" t="str">
-        <x:v>每相邻1件提琴声部道具，自身增加[10／13／17／21／25]人气，最多3件，不计自身</x:v>
+        <x:v>使相邻的其他提琴声部道具各增加[5／7／9／11／14]表演值，最多3件</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
@@ -3099,25 +3127,25 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="S17" s="43" t="n">
-        <x:v>13</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="T17" s="43" t="n">
-        <x:v>17</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="U17" s="43" t="n">
-        <x:v>21</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="V17" s="43" t="n">
-        <x:v>27</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="W17" s="43" t="n">
-        <x:v>33</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="X17" s="40" t="str">
-        <x:v>{"type":"count","scope":"adjacent","filter":{"category":["弦乐器"],"tag2":["现代"]},"cap":3,"excludeSource":true,"excludeAdjacent":false,"directions":[],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["现代"]},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y17" s="44" t="str">
-        <x:v>每相邻1件现代弦乐器，自身增加[13／17／21／27／33]人气，最多3件，不计自身</x:v>
+        <x:v>使相邻的现代乐器标签道具各增加[4／5／7／9／11]表演值，最多3件，不计自身</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
@@ -3177,25 +3205,25 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="S18" s="43" t="n">
-        <x:v>15</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="T18" s="43" t="n">
-        <x:v>20</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="U18" s="43" t="n">
-        <x:v>25</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="V18" s="43" t="n">
-        <x:v>31</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="W18" s="43" t="n">
-        <x:v>38</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="X18" s="40" t="str">
-        <x:v>{"type":"condition","clauses":[{"scope":"adjacent","filter":{"tag1":["提琴声部"]},"min":1,"max":null,"cap":1,"excludeSource":true,"directions":[]}],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["提琴声部"]},"cap":1,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y18" s="44" t="str">
-        <x:v>相邻至少1件提琴声部道具时，自身增加[15／20／25／31／38]人气；最多检查1件，不计自身</x:v>
+        <x:v>使相邻的1件其他提琴声部道具增加[7／9／12／14／18]表演值</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
@@ -3255,25 +3283,25 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="S19" s="43" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="T19" s="43" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="U19" s="43" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="V19" s="43" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="T19" s="43" t="n">
+      <x:c r="W19" s="43" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="U19" s="43" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="V19" s="43" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="W19" s="43" t="n">
-        <x:v>20</x:v>
-      </x:c>
       <x:c r="X19" s="40" t="str">
-        <x:v>{"type":"count","scope":"adjacent","filter":{"tag1":["拨弦声部"]},"cap":2,"excludeSource":true,"excludeAdjacent":false,"directions":[],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["拨弦声部"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y19" s="44" t="str">
-        <x:v>每相邻1件拨弦声部道具，自身增加[8／10／13／16／20]人气，最多2件，不计自身</x:v>
+        <x:v>使相邻的拨弦声部道具各增加[4／5／6／8／10]表演值，最多2件，不计自身</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
@@ -3348,10 +3376,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="X20" s="40" t="str">
-        <x:v>{"type":"count","scope":"global","filter":{"tag1":["拨弦声部"]},"cap":3,"excludeSource":true,"excludeAdjacent":false,"directions":[],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"global","filter":{"tag1":["拨弦声部"]},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y20" s="44" t="str">
-        <x:v>背包中每有1件拨弦声部道具，自身增加[3／4／5／6／8]人气，最多3件，不计自身</x:v>
+        <x:v>使背包中的其他拨弦声部道具各增加[3／4／5／6／8]表演值，最多3件</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="42" customHeight="1">
@@ -3411,25 +3439,25 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="S21" s="43" t="n">
-        <x:v>23</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="T21" s="43" t="n">
-        <x:v>30</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="U21" s="43" t="n">
-        <x:v>38</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="V21" s="43" t="n">
-        <x:v>47</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="W21" s="43" t="n">
-        <x:v>58</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="X21" s="40" t="str">
-        <x:v>{"type":"condition","clauses":[{"scope":"adjacent","filter":{"tag1":["提琴声部"]},"min":null,"max":0,"cap":null,"excludeSource":true,"directions":[]}],"recipient":"self"}</x:v>
+        <x:v>{"type":"condition","clauses":[{"scope":"adjacent","filter":{"tag1":["提琴声部"]},"min":null,"max":0,"cap":null,"excludeSource":true,"directions":[]}],"valueMode":"absolute","recipient":"self"}</x:v>
       </x:c>
       <x:c r="Y21" s="44" t="str">
-        <x:v>与其他提琴声部道具均不相邻时，自身增加[23／30／38／47／58]人气；检查全背包同类</x:v>
+        <x:v>与其他提琴声部道具均不相邻时，自身增加[10／13／17／21／25]表演值</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
@@ -3489,25 +3517,25 @@
         <x:v>148</x:v>
       </x:c>
       <x:c r="S22" s="43" t="n">
-        <x:v>47</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="T22" s="43" t="n">
-        <x:v>61</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="U22" s="43" t="n">
-        <x:v>77</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="V22" s="43" t="n">
-        <x:v>96</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="W22" s="43" t="n">
-        <x:v>117</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="X22" s="40" t="str">
-        <x:v>{"type":"balance","a":{"scope":"global","filter":{"tag1":["木管声部"]}},"b":{"scope":"global","filter":{"tag1":["铜管声部"]}},"minEach":2,"maxDiff":1,"capEach":4,"excludeSource":true,"recipient":"self"}</x:v>
+        <x:v>{"type":"balance","a":{"scope":"global","filter":{"tag1":["木管声部"]}},"b":{"scope":"global","filter":{"tag1":["铜管声部"]}},"minEach":2,"maxDiff":1,"capEach":4,"excludeSource":true,"valueMode":"percent","recipient":"self"}</x:v>
       </x:c>
       <x:c r="Y22" s="44" t="str">
-        <x:v>背包中木管声部与铜管声部道具数量差不超过1且各至少2件时，自身增加[47／61／77／96／117]人气；两组各最多计4件，不计自身</x:v>
+        <x:v>背包中木管声部与铜管声部数量差不超过1且各至少2件时，自身表演值增加[10／13／16／20／25]%</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
@@ -3567,25 +3595,25 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="S23" s="43" t="n">
-        <x:v>7</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="T23" s="43" t="n">
-        <x:v>12</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="U23" s="43" t="n">
-        <x:v>14</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="V23" s="43" t="n">
-        <x:v>16</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="W23" s="43" t="n">
-        <x:v>18</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="X23" s="40" t="str">
-        <x:v>{"type":"count","scope":"direction","filter":{"tag1":["木管声部"]},"cap":4,"excludeSource":true,"excludeAdjacent":false,"directions":["up","down"],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["木管声部"]},"cap":4,"excludeSource":true,"directions":["up","down"],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y23" s="44" t="str">
-        <x:v>上方与下方每有1件木管声部道具，自身增加[7／12／14／16／18]人气，两个方向合计最多4件，不计自身</x:v>
+        <x:v>使上方和下方的其他木管声部道具各增加[3／4／5／6／8]%表演值，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
@@ -3645,25 +3673,25 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="S24" s="43" t="n">
-        <x:v>30</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="T24" s="43" t="n">
-        <x:v>50</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="U24" s="43" t="n">
-        <x:v>58</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="V24" s="43" t="n">
-        <x:v>67</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="W24" s="43" t="n">
-        <x:v>75</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="X24" s="40" t="str">
-        <x:v>{"type":"condition","clauses":[{"scope":"direction","filter":{"tag1":["铜管声部"]},"min":1,"max":null,"cap":1,"excludeSource":true,"directions":["left"]},{"scope":"direction","filter":{"tag1":["铜管声部"]},"min":1,"max":null,"cap":1,"excludeSource":true,"directions":["right"]}],"recipient":"self"}</x:v>
+        <x:v>{"type":"groupBuff","clauses":[{"scope":"direction","filter":{"tag1":["铜管声部"]},"min":1,"max":null,"cap":null,"excludeSource":true,"directions":["left"]},{"scope":"direction","filter":{"tag1":["铜管声部"]},"min":1,"max":null,"cap":null,"excludeSource":true,"directions":["right"]}],"recipients":{"scope":"direction","directions":["left","right"],"filter":{"tag1":["铜管声部"]},"cap":4,"includeSource":false},"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y24" s="44" t="str">
-        <x:v>左侧与右侧各至少有1件铜管声部道具时，自身增加[30／50／58／67／75]人气；两侧各检查最多1件</x:v>
+        <x:v>左侧和右侧各至少有1件其他铜管声部道具时，使两侧符合条件的道具各增加[5／6／8／10／12]%表演值，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
@@ -3723,25 +3751,25 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S25" s="43" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="T25" s="43" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="U25" s="43" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="T25" s="43" t="n">
+      <x:c r="V25" s="43" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="U25" s="43" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="V25" s="43" t="n">
-        <x:v>16</x:v>
-      </x:c>
       <x:c r="W25" s="43" t="n">
-        <x:v>20</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="X25" s="40" t="str">
-        <x:v>{"type":"count","scope":"direction","filter":{"tag1":["木管声部"]},"cap":3,"excludeSource":true,"excludeAdjacent":false,"directions":["up"],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["木管声部"]},"cap":3,"excludeSource":true,"directions":["up"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y25" s="44" t="str">
-        <x:v>上方每有1件木管声部道具，自身增加[8／10／13／16／20]人气，最多3件，不计自身</x:v>
+        <x:v>使上方的其他木管声部道具各增加[5／6／8／10／12]表演值，最多3件</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="42" customHeight="1">
@@ -3801,25 +3829,25 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S26" s="43" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="T26" s="43" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="U26" s="43" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="T26" s="43" t="n">
+      <x:c r="V26" s="43" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="U26" s="43" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="V26" s="43" t="n">
-        <x:v>16</x:v>
-      </x:c>
       <x:c r="W26" s="43" t="n">
-        <x:v>20</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="X26" s="40" t="str">
-        <x:v>{"type":"count","scope":"direction","filter":{"tag1":["铜管声部"]},"cap":3,"excludeSource":true,"excludeAdjacent":false,"directions":["right"],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["铜管声部"]},"cap":3,"excludeSource":true,"directions":["right"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y26" s="44" t="str">
-        <x:v>右侧每有1件铜管声部道具，自身增加[8／10／13／16／20]人气，最多3件，不计自身</x:v>
+        <x:v>使右侧的其他铜管声部道具各增加[5／6／8／10／12]表演值，最多3件</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="42" customHeight="1">
@@ -3879,25 +3907,25 @@
         <x:v>75</x:v>
       </x:c>
       <x:c r="S27" s="43" t="n">
-        <x:v>8</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="T27" s="43" t="n">
-        <x:v>10</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="U27" s="43" t="n">
-        <x:v>13</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="V27" s="43" t="n">
-        <x:v>16</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="W27" s="43" t="n">
-        <x:v>20</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="X27" s="40" t="str">
-        <x:v>{"type":"count","scope":"global","filter":{"tag1":["木管声部"]},"cap":4,"excludeSource":true,"excludeAdjacent":false,"directions":[],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"global","filter":{"tag1":["木管声部"]},"cap":4,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y27" s="44" t="str">
-        <x:v>背包中每有1件木管声部道具，自身增加[8／10／13／16／20]人气，最多4件，不计自身</x:v>
+        <x:v>使背包中的其他木管声部道具各增加[4／5／7／9／11]表演值，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="42" customHeight="1">
@@ -3957,25 +3985,25 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="S28" s="43" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="T28" s="43" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="U28" s="43" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="V28" s="43" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="W28" s="43" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="T28" s="43" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="U28" s="43" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="V28" s="43" t="n">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="W28" s="43" t="n">
-        <x:v>25</x:v>
-      </x:c>
       <x:c r="X28" s="40" t="str">
-        <x:v>{"type":"count","scope":"direction","filter":{"tag1":["铜管声部"]},"cap":2,"excludeSource":true,"excludeAdjacent":false,"directions":["left"],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["铜管声部"]},"cap":2,"excludeSource":true,"directions":["left"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y28" s="44" t="str">
-        <x:v>左侧每有1件铜管声部道具，自身增加[10／13／17／21／25]人气，最多2件，不计自身</x:v>
+        <x:v>使左侧的其他铜管声部道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
@@ -4035,25 +4063,25 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="S29" s="43" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="T29" s="43" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="U29" s="43" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="T29" s="43" t="n">
+      <x:c r="V29" s="43" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="W29" s="43" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="U29" s="43" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="V29" s="43" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="W29" s="43" t="n">
-        <x:v>15</x:v>
-      </x:c>
       <x:c r="X29" s="40" t="str">
-        <x:v>{"type":"count","scope":"direction","filter":{"tag1":["木管声部"]},"cap":2,"excludeSource":true,"excludeAdjacent":false,"directions":["down"],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["木管声部"]},"cap":2,"excludeSource":true,"directions":["down"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y29" s="44" t="str">
-        <x:v>下方每有1件木管声部道具，自身增加[6／10／12／14／15]人气，最多2件，不计自身</x:v>
+        <x:v>使下方的其他木管声部道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="42" customHeight="1">
@@ -4113,25 +4141,25 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="S30" s="43" t="n">
-        <x:v>10</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="T30" s="43" t="n">
-        <x:v>16</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="U30" s="43" t="n">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="V30" s="43" t="n">
-        <x:v>22</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="W30" s="43" t="n">
-        <x:v>25</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="X30" s="40" t="str">
-        <x:v>{"type":"condition","clauses":[{"scope":"adjacent","filter":{"tag1":["铜管声部"]},"min":1,"max":null,"cap":1,"excludeSource":true,"directions":[]}],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["铜管声部"]},"cap":1,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y30" s="44" t="str">
-        <x:v>相邻至少1件铜管声部道具时，自身增加[10／16／19／22／25]人气；最多检查1件，不计自身</x:v>
+        <x:v>使相邻的1件其他铜管声部道具增加[7／9／12／14／18]表演值</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
@@ -4206,10 +4234,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="X31" s="40" t="str">
-        <x:v>{"type":"condition","clauses":[{"scope":"adjacent","filter":{"tag1":["木管声部"]},"min":null,"max":0,"cap":null,"excludeSource":true,"directions":[]}],"recipient":"self"}</x:v>
+        <x:v>{"type":"condition","clauses":[{"scope":"adjacent","filter":{"tag1":["木管声部"]},"min":null,"max":0,"cap":null,"excludeSource":true,"directions":[]}],"valueMode":"absolute","recipient":"self"}</x:v>
       </x:c>
       <x:c r="Y31" s="44" t="str">
-        <x:v>与其他木管声部道具均不相邻时，自身增加[10／13／17／21／25]人气；检查全背包同类</x:v>
+        <x:v>与其他木管声部道具均不相邻时，自身增加[10／13／17／21／25]表演值</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="42" customHeight="1">
@@ -4269,25 +4297,25 @@
         <x:v>195</x:v>
       </x:c>
       <x:c r="S32" s="43" t="n">
-        <x:v>22</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="T32" s="43" t="n">
-        <x:v>29</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="U32" s="43" t="n">
-        <x:v>36</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="V32" s="43" t="n">
-        <x:v>45</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="W32" s="43" t="n">
-        <x:v>55</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="X32" s="40" t="str">
-        <x:v>{"type":"count","scope":"adjacent","filter":{"tag1":["管弦打击"]},"cap":4,"excludeSource":true,"excludeAdjacent":false,"directions":[],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["管弦打击"]},"cap":4,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y32" s="44" t="str">
-        <x:v>每相邻1件管弦打击道具，自身增加[22／29／36／45／55]人气，最多4件，不计自身</x:v>
+        <x:v>使相邻的其他管弦打击道具各增加[4／5／6／8／10]%表演值，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
@@ -4347,25 +4375,25 @@
         <x:v>158</x:v>
       </x:c>
       <x:c r="S33" s="43" t="n">
-        <x:v>17</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="T33" s="43" t="n">
-        <x:v>22</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="U33" s="43" t="n">
-        <x:v>28</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="V33" s="43" t="n">
-        <x:v>35</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="W33" s="43" t="n">
-        <x:v>43</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="X33" s="40" t="str">
-        <x:v>{"type":"count","scope":"direction","filter":{"category":["打击乐器"]},"cap":4,"excludeSource":true,"excludeAdjacent":false,"directions":["up","down"],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["管弦打击"]},"cap":4,"excludeSource":true,"directions":["up","down"],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y33" s="44" t="str">
-        <x:v>上方与下方每有1件打击乐器，自身增加[17／22／28／35／43]人气，两个方向合计最多4件，不计自身</x:v>
+        <x:v>使上方和下方的其他管弦打击道具各增加[3／4／5／6／8]%表演值，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="42" customHeight="1">
@@ -4425,25 +4453,25 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="S34" s="43" t="n">
-        <x:v>13</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="T34" s="43" t="n">
-        <x:v>17</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="U34" s="43" t="n">
-        <x:v>21</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="V34" s="43" t="n">
-        <x:v>27</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="W34" s="43" t="n">
-        <x:v>33</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="X34" s="40" t="str">
-        <x:v>{"type":"count","scope":"direction","filter":{"tag1":["节奏打击"]},"cap":4,"excludeSource":true,"excludeAdjacent":false,"directions":["left","right"],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["节奏打击"]},"cap":4,"excludeSource":true,"directions":["left","right"],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y34" s="44" t="str">
-        <x:v>左侧与右侧每有1件节奏打击道具，自身增加[13／17／21／27／33]人气，两个方向合计最多4件，不计自身</x:v>
+        <x:v>使左侧和右侧的其他节奏打击道具各增加[3／4／5／6／8]%表演值，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="42" customHeight="1">
@@ -4503,25 +4531,25 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="S35" s="43" t="n">
-        <x:v>13</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="T35" s="43" t="n">
-        <x:v>17</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="U35" s="43" t="n">
-        <x:v>21</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="V35" s="43" t="n">
-        <x:v>27</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="W35" s="43" t="n">
-        <x:v>33</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="X35" s="40" t="str">
-        <x:v>{"type":"count","scope":"direction","filter":{"tag1":["管弦打击"]},"cap":3,"excludeSource":true,"excludeAdjacent":false,"directions":["down"],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["管弦打击"]},"cap":3,"excludeSource":true,"directions":["down"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y35" s="44" t="str">
-        <x:v>下方每有1件管弦打击道具，自身增加[13／17／21／27／33]人气，最多3件，不计自身</x:v>
+        <x:v>使下方的其他管弦打击道具各增加[5／7／9／11／14]表演值，最多3件</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="42" customHeight="1">
@@ -4581,25 +4609,25 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="S36" s="43" t="n">
-        <x:v>11</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="T36" s="43" t="n">
-        <x:v>14</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="U36" s="43" t="n">
-        <x:v>18</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="V36" s="43" t="n">
-        <x:v>23</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="W36" s="43" t="n">
-        <x:v>28</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="X36" s="40" t="str">
-        <x:v>{"type":"count","scope":"adjacent","filter":{"tag1":["管弦打击"]},"cap":3,"excludeSource":true,"excludeAdjacent":false,"directions":[],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["管弦打击"]},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y36" s="44" t="str">
-        <x:v>每相邻1件管弦打击道具，自身增加[11／14／18／23／28]人气，最多3件，不计自身</x:v>
+        <x:v>使相邻的其他管弦打击道具各增加[5／6／8／10／12]表演值，最多3件</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="42" customHeight="1">
@@ -4659,25 +4687,25 @@
         <x:v>75</x:v>
       </x:c>
       <x:c r="S37" s="43" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="T37" s="43" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="U37" s="43" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="V37" s="43" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="T37" s="43" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="U37" s="43" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="V37" s="43" t="n">
-        <x:v>21</x:v>
-      </x:c>
       <x:c r="W37" s="43" t="n">
-        <x:v>25</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="X37" s="40" t="str">
-        <x:v>{"type":"count","scope":"direction","filter":{"tag1":["节奏打击"]},"cap":3,"excludeSource":true,"excludeAdjacent":false,"directions":["left"],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["节奏打击"]},"cap":3,"excludeSource":true,"directions":["left"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y37" s="44" t="str">
-        <x:v>左侧每有1件节奏打击道具，自身增加[10／13／17／21／25]人气，最多3件，不计自身</x:v>
+        <x:v>使左侧的其他节奏打击道具各增加[5／6／8／10／12]表演值，最多3件</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="42" customHeight="1">
@@ -4737,25 +4765,25 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="S38" s="43" t="n">
-        <x:v>13</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="T38" s="43" t="n">
-        <x:v>17</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="U38" s="43" t="n">
-        <x:v>21</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="V38" s="43" t="n">
-        <x:v>27</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="W38" s="43" t="n">
-        <x:v>33</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="X38" s="40" t="str">
-        <x:v>{"type":"condition","clauses":[{"scope":"adjacent","filter":{"tag1":["管弦打击"]},"min":1,"max":null,"cap":1,"excludeSource":true,"directions":[]}],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["管弦打击"]},"cap":1,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y38" s="44" t="str">
-        <x:v>相邻至少1件管弦打击道具时，自身增加[13／17／21／27／33]人气；最多检查1件，不计自身</x:v>
+        <x:v>使相邻的1件其他管弦打击道具增加[7／9／12／14／18]表演值</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="42" customHeight="1">
@@ -4815,25 +4843,25 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="S39" s="43" t="n">
-        <x:v>15</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="T39" s="43" t="n">
-        <x:v>20</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="U39" s="43" t="n">
-        <x:v>25</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="V39" s="43" t="n">
-        <x:v>31</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="W39" s="43" t="n">
-        <x:v>38</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="X39" s="40" t="str">
-        <x:v>{"type":"condition","clauses":[{"scope":"adjacent","filter":{"tag1":["节奏打击"]},"min":1,"max":null,"cap":1,"excludeSource":true,"directions":[]}],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["节奏打击"]},"cap":1,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y39" s="44" t="str">
-        <x:v>相邻至少1件节奏打击道具时，自身增加[15／20／25／31／38]人气；最多检查1件，不计自身</x:v>
+        <x:v>使相邻的1件其他节奏打击道具增加[7／9／12／14／18]表演值</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="42" customHeight="1">
@@ -4908,10 +4936,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="X40" s="40" t="str">
-        <x:v>{"type":"count","scope":"adjacent","filter":{"category":["打击乐器"]},"cap":2,"excludeSource":true,"excludeAdjacent":false,"directions":[],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["管弦打击","节奏打击"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y40" s="44" t="str">
-        <x:v>每相邻1件打击乐器，自身增加[3／4／5／6／8]人气，最多2件，不计自身</x:v>
+        <x:v>使相邻的其他管弦打击或节奏打击道具各增加[3／4／5／6／8]表演值，最多2件</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="42" customHeight="1">
@@ -4986,10 +5014,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="X41" s="40" t="str">
-        <x:v>{"type":"condition","clauses":[{"scope":"adjacent","filter":{"tag1":["节奏打击"]},"min":null,"max":0,"cap":null,"excludeSource":true,"directions":[]}],"recipient":"self"}</x:v>
+        <x:v>{"type":"condition","clauses":[{"scope":"adjacent","filter":{"tag1":["节奏打击"]},"min":null,"max":0,"cap":null,"excludeSource":true,"directions":[]}],"valueMode":"absolute","recipient":"self"}</x:v>
       </x:c>
       <x:c r="Y41" s="44" t="str">
-        <x:v>与其他节奏打击道具均不相邻时，自身增加[10／13／17／21／25]人气；检查全背包同类</x:v>
+        <x:v>与其他节奏打击道具均不相邻时，自身增加[10／13／17／21／25]表演值</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="42" customHeight="1">
@@ -5049,25 +5077,25 @@
         <x:v>148</x:v>
       </x:c>
       <x:c r="S42" s="43" t="n">
-        <x:v>11</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="T42" s="43" t="n">
-        <x:v>14</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="U42" s="43" t="n">
-        <x:v>18</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="V42" s="43" t="n">
-        <x:v>23</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="W42" s="43" t="n">
-        <x:v>28</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="X42" s="40" t="str">
-        <x:v>{"type":"groupBuff","clauses":[{"scope":"global","filter":{"tag1":["芭蕾服装"]},"min":2,"max":null,"cap":null,"excludeSource":false,"directions":[]},{"scope":"global","filter":{"category":["舞台装饰"],"tag2":["古典"]},"min":2,"max":null,"cap":null,"excludeSource":true,"directions":[]}],"recipients":{"filter":{"tag1":["芭蕾服装"]},"cap":4,"includeSource":true}}</x:v>
+        <x:v>{"type":"targetBuff","scope":"global","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["古典"]},"cap":6,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y42" s="44" t="str">
-        <x:v>背包中芭蕾服装与古典舞台装饰各至少2件时，每件芭蕾服装增加[11／14／18／23／28]人气；阈值统计包含自身，受益目标包含自身，最多作用4件芭蕾服装，同一目标结算1次</x:v>
+        <x:v>使背包中的古典乐器标签道具各增加[3／4／5／6／8]%表演值，最多6件</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="42" customHeight="1">
@@ -5127,25 +5155,25 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="S43" s="43" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="T43" s="43" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="U43" s="43" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="V43" s="43" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="W43" s="43" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="T43" s="43" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="U43" s="43" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="V43" s="43" t="n">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="W43" s="43" t="n">
-        <x:v>25</x:v>
-      </x:c>
       <x:c r="X43" s="40" t="str">
-        <x:v>{"type":"count","scope":"adjacent","filter":{"tag1":["芭蕾服装"]},"cap":3,"excludeSource":true,"excludeAdjacent":false,"directions":[],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["提琴声部"]},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y43" s="44" t="str">
-        <x:v>每相邻1件芭蕾服装，自身增加[10／13／17／21／25]人气，最多3件，不计自身</x:v>
+        <x:v>使相邻的提琴声部道具各增加[4／5／6／8／10]%表演值，最多3件</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="42" customHeight="1">
@@ -5205,25 +5233,25 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="S44" s="43" t="n">
-        <x:v>17</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="T44" s="43" t="n">
-        <x:v>22</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="U44" s="43" t="n">
-        <x:v>28</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="V44" s="43" t="n">
-        <x:v>35</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="W44" s="43" t="n">
-        <x:v>43</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="X44" s="40" t="str">
-        <x:v>{"type":"count","scope":"adjacent","filter":{"tag1":["歌剧服装"]},"cap":3,"excludeSource":true,"excludeAdjacent":false,"directions":[],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["古典"]},"cap":4,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y44" s="44" t="str">
-        <x:v>每相邻1件歌剧服装，自身增加[17／22／28／35／43]人气，最多3件，不计自身</x:v>
+        <x:v>使相邻的古典乐器标签道具各增加[3／4／5／6／8]%表演值，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="42" customHeight="1">
@@ -5283,25 +5311,25 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="S45" s="43" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="T45" s="43" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="U45" s="43" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="T45" s="43" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="U45" s="43" t="n">
-        <x:v>20</x:v>
-      </x:c>
       <x:c r="V45" s="43" t="n">
-        <x:v>25</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="W45" s="43" t="n">
-        <x:v>30</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="X45" s="40" t="str">
-        <x:v>{"type":"condition","clauses":[{"scope":"adjacent","filter":{"tag1":["爵士服装"]},"min":null,"max":0,"cap":null,"excludeSource":true,"directions":[]}],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["现代"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y45" s="44" t="str">
-        <x:v>与其他爵士服装均不相邻时，自身增加[12／16／20／25／30]人气；检查全背包同类</x:v>
+        <x:v>使相邻的现代乐器标签道具各增加[7／9／12／14／18]表演值，最多2件</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="42" customHeight="1">
@@ -5361,25 +5389,25 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="S46" s="43" t="n">
-        <x:v>13</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="T46" s="43" t="n">
-        <x:v>17</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="U46" s="43" t="n">
-        <x:v>21</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="V46" s="43" t="n">
-        <x:v>27</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="W46" s="43" t="n">
-        <x:v>33</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="X46" s="40" t="str">
-        <x:v>{"type":"count","scope":"global","filter":{"tag1":["歌剧服装"]},"cap":3,"excludeSource":true,"excludeAdjacent":false,"directions":[],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"global","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["古典"]},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y46" s="44" t="str">
-        <x:v>背包中每有1件其他歌剧服装，自身增加[13／17／21／27／33]人气，最多3件，不计自身</x:v>
+        <x:v>使背包中的古典乐器标签道具各增加[5／6／8／10／12]表演值，最多3件</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="42" customHeight="1">
@@ -5439,25 +5467,25 @@
         <x:v>75</x:v>
       </x:c>
       <x:c r="S47" s="43" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="T47" s="43" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="U47" s="43" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="V47" s="43" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="T47" s="43" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="U47" s="43" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="V47" s="43" t="n">
-        <x:v>21</x:v>
-      </x:c>
       <x:c r="W47" s="43" t="n">
-        <x:v>25</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="X47" s="40" t="str">
-        <x:v>{"type":"count","scope":"direction","filter":{"tag1":["爵士服装"]},"cap":3,"excludeSource":true,"excludeAdjacent":false,"directions":["left","right"],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["现代"]},"cap":3,"excludeSource":true,"directions":["left","right"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y47" s="44" t="str">
-        <x:v>左侧与右侧每有1件爵士服装，自身增加[10／13／17／21／25]人气，两个方向合计最多3件，不计自身</x:v>
+        <x:v>使左侧和右侧的现代乐器标签道具各增加[5／6／8／10／12]表演值，最多3件</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="42" customHeight="1">
@@ -5517,25 +5545,25 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="S48" s="43" t="n">
-        <x:v>11</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="T48" s="43" t="n">
-        <x:v>14</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="U48" s="43" t="n">
-        <x:v>18</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="V48" s="43" t="n">
-        <x:v>23</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="W48" s="43" t="n">
-        <x:v>28</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="X48" s="40" t="str">
-        <x:v>{"type":"condition","clauses":[{"scope":"adjacent","filter":{"tag1":["芭蕾服装"]},"min":1,"max":null,"cap":1,"excludeSource":true,"directions":[]}],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["提琴声部"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y48" s="44" t="str">
-        <x:v>相邻至少1件芭蕾服装时，自身增加[11／14／18／23／28]人气；最多检查1件，不计自身</x:v>
+        <x:v>使相邻的提琴声部道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="42" customHeight="1">
@@ -5610,10 +5638,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="X49" s="40" t="str">
-        <x:v>{"type":"count","scope":"adjacent","filter":{"tag1":["芭蕾服装"]},"cap":2,"excludeSource":true,"excludeAdjacent":false,"directions":[],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["提琴声部"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y49" s="44" t="str">
-        <x:v>每相邻1件芭蕾服装，自身增加[3／4／5／6／8]人气，最多2件，不计自身</x:v>
+        <x:v>使相邻的提琴声部道具各增加[3／4／5／6／8]表演值，最多2件</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="42" customHeight="1">
@@ -5679,7 +5707,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="U50" s="43" t="n">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="V50" s="43" t="n">
         <x:v>8</x:v>
@@ -5688,10 +5716,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="X50" s="40" t="str">
-        <x:v>{"type":"count","scope":"global","filter":{"tag1":["歌剧服装"]},"cap":2,"excludeSource":true,"excludeAdjacent":false,"directions":[],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"global","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["古典"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y50" s="44" t="str">
-        <x:v>背包中每有1件其他歌剧服装，自身增加[4／5／7／8／10]人气，最多2件，不计自身</x:v>
+        <x:v>使背包中的古典乐器标签道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="42" customHeight="1">
@@ -5751,25 +5779,25 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="S51" s="43" t="n">
-        <x:v>9</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="T51" s="43" t="n">
-        <x:v>12</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="U51" s="43" t="n">
-        <x:v>15</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="V51" s="43" t="n">
-        <x:v>18</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="W51" s="43" t="n">
-        <x:v>23</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="X51" s="40" t="str">
-        <x:v>{"type":"condition","clauses":[{"scope":"adjacent","filter":{"tag1":["爵士服装"]},"min":1,"max":null,"cap":1,"excludeSource":true,"directions":[]}],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["现代"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y51" s="44" t="str">
-        <x:v>相邻至少1件爵士服装时，自身增加[9／12／15／18／23]人气；最多检查1件，不计自身</x:v>
+        <x:v>使相邻的现代乐器标签道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="42" customHeight="1">
@@ -5829,25 +5857,25 @@
         <x:v>308</x:v>
       </x:c>
       <x:c r="S52" s="43" t="n">
-        <x:v>158</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="T52" s="43" t="n">
-        <x:v>194</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="U52" s="43" t="n">
-        <x:v>230</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="V52" s="43" t="n">
-        <x:v>266</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="W52" s="43" t="n">
-        <x:v>394</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="X52" s="40" t="str">
-        <x:v>{"type":"balance","a":{"scope":"global","filter":{"category":["服装"],"tag2":["古典"]}},"b":{"scope":"global","filter":{"category":["舞台装饰"],"tag2":["古典"]}},"minEach":2,"maxDiff":1,"capEach":4,"excludeSource":true,"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"global","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["古典"]},"cap":6,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y52" s="44" t="str">
-        <x:v>背包中古典服装与古典舞台装饰数量差不超过1且各至少2件时，自身增加[158／194／230／266／394]人气；两组各最多计4件，不计自身</x:v>
+        <x:v>使背包中的古典乐器标签道具各增加[4／5／6／8／10]%表演值，最多6件</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="42" customHeight="1">
@@ -5907,25 +5935,25 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="S53" s="43" t="n">
-        <x:v>62</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="T53" s="43" t="n">
-        <x:v>81</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="U53" s="43" t="n">
-        <x:v>102</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="V53" s="43" t="n">
-        <x:v>127</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="W53" s="43" t="n">
-        <x:v>155</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="X53" s="40" t="str">
-        <x:v>{"type":"balance","a":{"scope":"direction","directions":["left"],"filter":{"tag1":["灯光"]}},"b":{"scope":"direction","directions":["right"],"filter":{"tag1":["布景"]}},"minEach":1,"maxDiff":0,"capEach":3,"excludeSource":true,"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"]},"cap":4,"excludeSource":true,"directions":["left","right"],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y53" s="44" t="str">
-        <x:v>左侧灯光与右侧布景数量相等且各至少1件时，自身增加[62／81／102／127／155]人气；两侧各最多计3件，不计自身</x:v>
+        <x:v>使左侧和右侧的乐器标签道具各增加[3／4／5／6／8]%表演值，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="42" customHeight="1">
@@ -5985,25 +6013,25 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="S54" s="43" t="n">
-        <x:v>58</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="T54" s="43" t="n">
-        <x:v>75</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="U54" s="43" t="n">
-        <x:v>96</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="V54" s="43" t="n">
-        <x:v>119</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="W54" s="43" t="n">
-        <x:v>145</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="X54" s="40" t="str">
-        <x:v>{"type":"condition","clauses":[{"scope":"global","filter":{"tag1":["布景"]},"min":2,"max":null,"cap":3,"excludeSource":true,"directions":[]},{"scope":"global","filter":{"tag1":["声场"]},"min":2,"max":null,"cap":3,"excludeSource":true,"directions":[]}],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"global","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"minArea":4},"cap":4,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y54" s="44" t="str">
-        <x:v>背包中布景与声场道具各至少2件时，自身增加[58／75／96／119／145]人气；两类各最多计3件，不计自身</x:v>
+        <x:v>使背包中占用4格及以上的乐器标签道具各增加[4／5／6／8／10]%表演值，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="42" customHeight="1">
@@ -6063,25 +6091,25 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S55" s="43" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="T55" s="43" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="U55" s="43" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="T55" s="43" t="n">
+      <x:c r="V55" s="43" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="U55" s="43" t="n">
+      <x:c r="W55" s="43" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="V55" s="43" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="W55" s="43" t="n">
-        <x:v>15</x:v>
-      </x:c>
       <x:c r="X55" s="40" t="str">
-        <x:v>{"type":"count","scope":"direction","filter":{"any":true},"cap":4,"excludeSource":true,"excludeAdjacent":false,"directions":["up"],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"]},"cap":4,"excludeSource":true,"directions":["up"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y55" s="44" t="str">
-        <x:v>上方每有1件道具，自身增加[6／8／10／12／15]人气，最多4件</x:v>
+        <x:v>使上方的乐器标签道具各增加[4／5／6／8／10]表演值，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="42" customHeight="1">
@@ -6141,25 +6169,25 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S56" s="43" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="T56" s="43" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="U56" s="43" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="T56" s="43" t="n">
+      <x:c r="V56" s="43" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="U56" s="43" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="V56" s="43" t="n">
-        <x:v>16</x:v>
-      </x:c>
       <x:c r="W56" s="43" t="n">
-        <x:v>20</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="X56" s="40" t="str">
-        <x:v>{"type":"count","scope":"direction","filter":{"tag1":["布景"]},"cap":3,"excludeSource":true,"excludeAdjacent":false,"directions":["left","right"],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["古典"]},"cap":3,"excludeSource":true,"directions":["left","right"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y56" s="44" t="str">
-        <x:v>左侧与右侧每有1件布景，自身增加[8／10／13／16／20]人气，两个方向合计最多3件，不计自身</x:v>
+        <x:v>使左侧和右侧的古典乐器标签道具各增加[5／6／8／10／12]表演值，最多3件</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="42" customHeight="1">
@@ -6219,25 +6247,25 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="S57" s="43" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="T57" s="43" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="U57" s="43" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="T57" s="43" t="n">
+      <x:c r="V57" s="43" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="U57" s="43" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="V57" s="43" t="n">
-        <x:v>16</x:v>
-      </x:c>
       <x:c r="W57" s="43" t="n">
-        <x:v>20</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="X57" s="40" t="str">
-        <x:v>{"type":"count","scope":"global","filter":{"tag1":["声场"]},"cap":3,"excludeSource":true,"excludeAdjacent":false,"directions":[],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"global","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"]},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y57" s="44" t="str">
-        <x:v>背包中每有1件其他声场道具，自身增加[8／10／13／16／20]人气，最多3件，不计自身</x:v>
+        <x:v>使背包中的乐器标签道具各增加[5／6／8／10／12]表演值，最多3件</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="42" customHeight="1">
@@ -6297,25 +6325,25 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="S58" s="43" t="n">
-        <x:v>15</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="T58" s="43" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="U58" s="43" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="V58" s="43" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="W58" s="43" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="U58" s="43" t="n">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="V58" s="43" t="n">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="W58" s="43" t="n">
-        <x:v>38</x:v>
-      </x:c>
       <x:c r="X58" s="40" t="str">
-        <x:v>{"type":"condition","clauses":[{"scope":"adjacent","filter":{"tag1":["灯光"]},"min":1,"max":null,"cap":1,"excludeSource":true,"directions":[]}],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["现代"]},"cap":1,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y58" s="44" t="str">
-        <x:v>相邻至少1件灯光时，自身增加[15／20／25／31／38]人气；最多检查1件，不计自身</x:v>
+        <x:v>使相邻的1件现代乐器标签道具增加[8／10／13／16／20]表演值</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="42" customHeight="1">
@@ -6375,25 +6403,25 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="S59" s="43" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="T59" s="43" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="U59" s="43" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="V59" s="43" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="T59" s="43" t="n">
+      <x:c r="W59" s="43" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="U59" s="43" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="V59" s="43" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="W59" s="43" t="n">
-        <x:v>20</x:v>
-      </x:c>
       <x:c r="X59" s="40" t="str">
-        <x:v>{"type":"count","scope":"adjacent","filter":{"tag1":["布景"]},"cap":2,"excludeSource":true,"excludeAdjacent":false,"directions":[],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["古典"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y59" s="44" t="str">
-        <x:v>每相邻1件布景，自身增加[8／10／13／16／20]人气，最多2件，不计自身</x:v>
+        <x:v>使相邻的古典乐器标签道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="42" customHeight="1">
@@ -6453,25 +6481,25 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="S60" s="43" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="T60" s="43" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="T60" s="43" t="n">
+      <x:c r="U60" s="43" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="U60" s="43" t="n">
-        <x:v>17</x:v>
-      </x:c>
       <x:c r="V60" s="43" t="n">
-        <x:v>21</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="W60" s="43" t="n">
-        <x:v>25</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="X60" s="40" t="str">
-        <x:v>{"type":"condition","clauses":[{"scope":"adjacent","filter":{"tag1":["灯光"]},"min":null,"max":0,"cap":null,"excludeSource":true,"directions":[]}],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"]},"cap":1,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y60" s="44" t="str">
-        <x:v>与其他灯光均不相邻时，自身增加[10／13／17／21／25]人气；检查全背包同类</x:v>
+        <x:v>使相邻的1件乐器标签道具增加[8／10／13／16／20]表演值</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="42" customHeight="1">
@@ -6537,7 +6565,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="U61" s="45" t="n">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="V61" s="45" t="n">
         <x:v>8</x:v>
@@ -6546,10 +6574,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="X61" s="42" t="str">
-        <x:v>{"type":"count","scope":"global","filter":{"tag1":["声场"]},"cap":2,"excludeSource":true,"excludeAdjacent":false,"directions":[],"recipient":"self"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"global","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y61" s="46" t="str">
-        <x:v>背包中每有1件其他声场道具，自身增加[4／5／7／8／10]人气，最多2件，不计自身</x:v>
+        <x:v>使背包中的乐器标签道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6564,7 +6592,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6563558ebca4d1a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a478579b2a0494e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Use categories for all prop effects
</commit_message>
<xml_diff>
--- a/data/爱乐之城-表演道具验证配置.xlsx
+++ b/data/爱乐之城-表演道具验证配置.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="Rd97b1f70421d45c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规则配置" sheetId="2" r:id="Rd81a7ed8725f4157"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品质配置" sheetId="3" r:id="R75fc9848daab41e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表演规则" sheetId="4" r:id="R5f1b896861f947d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发挥档位" sheetId="5" r:id="R3526c4e186b24d73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="现场事件" sheetId="6" r:id="R74a43003582a4165"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="种类表演特性" sheetId="7" r:id="R7b660783b5b54f54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="道具配置" sheetId="8" r:id="R6f862d8f5aa24bc1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="Rf6aa04f23adf40af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规则配置" sheetId="2" r:id="R1523c91b6fda4258"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品质配置" sheetId="3" r:id="Ra90f1dd1ffb64614"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表演规则" sheetId="4" r:id="Rc3a89a1fefb1485b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发挥档位" sheetId="5" r:id="R018addef3cc84a45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="现场事件" sheetId="6" r:id="R87b36c9f54f34505"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="种类表演特性" sheetId="7" r:id="Rc28ec5b0a231472d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="道具配置" sheetId="8" r:id="Rb20424eff1324042"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -975,7 +975,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e14deed53be46d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d5aea9d26fb4eb3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1079,7 +1079,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re69cb55fc2324f5c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02dbce2d04744fb8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1287,7 +1287,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra19878cdde9143c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb379907417324fb6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1407,7 +1407,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1536f8f27aa4162"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78a84dd9ad0f4a8c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1649,7 +1649,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R707dd46217fc488f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf0eff2bc0c44115"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1787,7 +1787,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R300ff96c92c34fe8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cef766f5ee64516"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1911,7 +1911,7 @@
         <x:v>键盘乐器</x:v>
       </x:c>
       <x:c r="D2" s="40" t="str">
-        <x:v>管风琴键盘</x:v>
+        <x:v>键盘乐器</x:v>
       </x:c>
       <x:c r="E2" s="40" t="str">
         <x:v>古典</x:v>
@@ -1972,10 +1972,10 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="X2" s="40" t="str">
-        <x:v>{"type":"condition","clauses":[{"scope":"global","filter":{"tag1":["提琴声部"]},"min":1,"max":null,"cap":null,"excludeSource":true,"directions":[]},{"scope":"global","filter":{"tag1":["木管声部"]},"min":1,"max":null,"cap":null,"excludeSource":true,"directions":[]},{"scope":"global","filter":{"tag1":["管弦打击"]},"min":1,"max":null,"cap":null,"excludeSource":true,"directions":[]}],"valueMode":"percent","recipient":"self"}</x:v>
+        <x:v>{"type":"condition","clauses":[{"scope":"global","filter":{"category":["弦乐器"]},"min":1,"max":null,"cap":null,"excludeSource":true,"directions":[]},{"scope":"global","filter":{"category":["管乐器"]},"min":1,"max":null,"cap":null,"excludeSource":true,"directions":[]},{"scope":"global","filter":{"category":["打击乐器"]},"min":1,"max":null,"cap":null,"excludeSource":true,"directions":[]}],"valueMode":"percent","recipient":"self"}</x:v>
       </x:c>
       <x:c r="Y2" s="44" t="str">
-        <x:v>背包中提琴声部、木管声部和管弦打击各至少1件时，自身表演值增加[12／15／19／24／30]%</x:v>
+        <x:v>背包中弦乐器、管乐器和打击乐器各至少1件时，自身表演值增加[12／15／19／24／30]%</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
@@ -1989,7 +1989,7 @@
         <x:v>键盘乐器</x:v>
       </x:c>
       <x:c r="D3" s="40" t="str">
-        <x:v>钢琴键盘</x:v>
+        <x:v>键盘乐器</x:v>
       </x:c>
       <x:c r="E3" s="40" t="str">
         <x:v>古典</x:v>
@@ -2050,10 +2050,10 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="X3" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["古典"]},"cap":4,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"category":["键盘乐器","弦乐器","管乐器","打击乐器"]},"cap":4,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y3" s="44" t="str">
-        <x:v>使相邻的古典乐器标签道具各增加[5／6／8／10／12]%表演值，最多4件</x:v>
+        <x:v>使相邻的乐器道具各增加[5／6／8／10／12]%表演值，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
@@ -2067,7 +2067,7 @@
         <x:v>键盘乐器</x:v>
       </x:c>
       <x:c r="D4" s="40" t="str">
-        <x:v>管风琴键盘</x:v>
+        <x:v>键盘乐器</x:v>
       </x:c>
       <x:c r="E4" s="40" t="str">
         <x:v>古典</x:v>
@@ -2128,10 +2128,10 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="X4" s="40" t="str">
-        <x:v>{"type":"groupBuff","clauses":[{"scope":"direction","filter":{"tag1":["提琴声部","拨弦声部"]},"min":1,"max":null,"cap":null,"excludeSource":true,"directions":["left"]},{"scope":"direction","filter":{"tag1":["木管声部","铜管声部"]},"min":1,"max":null,"cap":null,"excludeSource":true,"directions":["right"]}],"recipients":{"scope":"direction","directions":["left","right"],"filter":{"tag1":["提琴声部","拨弦声部","木管声部","铜管声部"]},"cap":4,"includeSource":false},"valueMode":"percent"}</x:v>
+        <x:v>{"type":"groupBuff","clauses":[{"scope":"direction","filter":{"category":["弦乐器"]},"min":1,"max":null,"cap":null,"excludeSource":true,"directions":["left"]},{"scope":"direction","filter":{"category":["管乐器"]},"min":1,"max":null,"cap":null,"excludeSource":true,"directions":["right"]}],"recipients":{"scope":"direction","directions":["left","right"],"filter":{"category":["弦乐器","管乐器"]},"cap":4,"includeSource":false},"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y4" s="44" t="str">
-        <x:v>左侧至少有1件提琴声部或拨弦声部，且右侧至少有1件木管声部或铜管声部时，使两侧符合条件的道具各增加[5／6／8／10／12]%表演值，最多4件</x:v>
+        <x:v>左侧至少有1件弦乐器，且右侧至少有1件管乐器时，使两侧符合条件的道具各增加[5／6／8／10／12]%表演值，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="42" customHeight="1">
@@ -2145,7 +2145,7 @@
         <x:v>键盘乐器</x:v>
       </x:c>
       <x:c r="D5" s="40" t="str">
-        <x:v>钢琴键盘</x:v>
+        <x:v>键盘乐器</x:v>
       </x:c>
       <x:c r="E5" s="40" t="str">
         <x:v>现代</x:v>
@@ -2206,10 +2206,10 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="X5" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"]},"cap":4,"excludeSource":true,"directions":["up","down"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"category":["键盘乐器","弦乐器","管乐器","打击乐器"]},"cap":4,"excludeSource":true,"directions":["up","down"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y5" s="44" t="str">
-        <x:v>使上方和下方的乐器标签道具各增加[5／7／9／11／14]表演值，最多4件</x:v>
+        <x:v>使上方和下方的乐器道具各增加[5／7／9／11／14]表演值，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
@@ -2223,7 +2223,7 @@
         <x:v>键盘乐器</x:v>
       </x:c>
       <x:c r="D6" s="40" t="str">
-        <x:v>管风琴键盘</x:v>
+        <x:v>键盘乐器</x:v>
       </x:c>
       <x:c r="E6" s="40" t="str">
         <x:v>现代</x:v>
@@ -2284,10 +2284,10 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="X6" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"global","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["现代"]},"cap":4,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"global","filter":{"category":["键盘乐器","弦乐器","管乐器","打击乐器"]},"cap":4,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y6" s="44" t="str">
-        <x:v>使背包中的现代乐器标签道具各增加[5／7／9／11／14]表演值，最多4件，不计自身</x:v>
+        <x:v>使背包中的乐器道具各增加[5／7／9／11／14]表演值，最多4件，不计自身</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
@@ -2301,7 +2301,7 @@
         <x:v>键盘乐器</x:v>
       </x:c>
       <x:c r="D7" s="40" t="str">
-        <x:v>钢琴键盘</x:v>
+        <x:v>键盘乐器</x:v>
       </x:c>
       <x:c r="E7" s="40" t="str">
         <x:v>古典</x:v>
@@ -2362,10 +2362,10 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="X7" s="40" t="str">
-        <x:v>{"type":"condition","clauses":[{"scope":"adjacent","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"]},"min":null,"max":2,"cap":null,"excludeSource":true,"directions":[]}],"valueMode":"absolute","recipient":"self"}</x:v>
+        <x:v>{"type":"condition","clauses":[{"scope":"adjacent","filter":{"category":["键盘乐器","弦乐器","管乐器","打击乐器"]},"min":null,"max":2,"cap":null,"excludeSource":true,"directions":[]}],"valueMode":"absolute","recipient":"self"}</x:v>
       </x:c>
       <x:c r="Y7" s="44" t="str">
-        <x:v>相邻的乐器标签道具不超过2件时，自身增加[38／49／63／78／95]表演值</x:v>
+        <x:v>相邻的乐器道具不超过2件时，自身增加[38／49／63／78／95]表演值</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
@@ -2379,7 +2379,7 @@
         <x:v>键盘乐器</x:v>
       </x:c>
       <x:c r="D8" s="40" t="str">
-        <x:v>钢琴键盘</x:v>
+        <x:v>键盘乐器</x:v>
       </x:c>
       <x:c r="E8" s="40" t="str">
         <x:v>古典</x:v>
@@ -2440,10 +2440,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="X8" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"category":["键盘乐器","弦乐器","管乐器","打击乐器"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y8" s="44" t="str">
-        <x:v>使相邻的乐器标签道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
+        <x:v>使相邻的乐器道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
@@ -2457,7 +2457,7 @@
         <x:v>键盘乐器</x:v>
       </x:c>
       <x:c r="D9" s="40" t="str">
-        <x:v>管风琴键盘</x:v>
+        <x:v>键盘乐器</x:v>
       </x:c>
       <x:c r="E9" s="40" t="str">
         <x:v>现代</x:v>
@@ -2518,10 +2518,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="X9" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"]},"cap":2,"excludeSource":true,"directions":["left"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"category":["键盘乐器","弦乐器","管乐器","打击乐器"]},"cap":2,"excludeSource":true,"directions":["left"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y9" s="44" t="str">
-        <x:v>使左侧的乐器标签道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
+        <x:v>使左侧的乐器道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
@@ -2535,7 +2535,7 @@
         <x:v>键盘乐器</x:v>
       </x:c>
       <x:c r="D10" s="40" t="str">
-        <x:v>钢琴键盘</x:v>
+        <x:v>键盘乐器</x:v>
       </x:c>
       <x:c r="E10" s="40" t="str">
         <x:v>古典</x:v>
@@ -2596,10 +2596,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="X10" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"global","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"minArea":4},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"global","filter":{"minArea":4,"category":["键盘乐器","弦乐器","管乐器","打击乐器"]},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y10" s="44" t="str">
-        <x:v>使背包中占用4格及以上的乐器标签道具各增加[4／5／6／8／10]表演值，最多3件，不计自身</x:v>
+        <x:v>使背包中占用4格及以上的乐器道具各增加[4／5／6／8／10]表演值，最多3件，不计自身</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
@@ -2613,7 +2613,7 @@
         <x:v>键盘乐器</x:v>
       </x:c>
       <x:c r="D11" s="40" t="str">
-        <x:v>管风琴键盘</x:v>
+        <x:v>键盘乐器</x:v>
       </x:c>
       <x:c r="E11" s="40" t="str">
         <x:v>古典</x:v>
@@ -2674,10 +2674,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="X11" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"]},"cap":2,"excludeSource":true,"directions":["right"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"category":["键盘乐器","弦乐器","管乐器","打击乐器"]},"cap":2,"excludeSource":true,"directions":["right"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y11" s="44" t="str">
-        <x:v>使右侧的乐器标签道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
+        <x:v>使右侧的乐器道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
@@ -2691,7 +2691,7 @@
         <x:v>弦乐器</x:v>
       </x:c>
       <x:c r="D12" s="40" t="str">
-        <x:v>拨弦声部</x:v>
+        <x:v>弦乐器</x:v>
       </x:c>
       <x:c r="E12" s="40" t="str">
         <x:v>古典</x:v>
@@ -2752,10 +2752,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="X12" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"global","filter":{"tag1":["提琴声部"]},"cap":6,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"global","filter":{"category":["弦乐器"]},"cap":6,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y12" s="44" t="str">
-        <x:v>使背包中的提琴声部道具各增加[3／4／5／6／8]%表演值，最多6件</x:v>
+        <x:v>使背包中的弦乐器道具各增加[3／4／5／6／8]%表演值，最多6件</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
@@ -2769,7 +2769,7 @@
         <x:v>弦乐器</x:v>
       </x:c>
       <x:c r="D13" s="40" t="str">
-        <x:v>提琴声部</x:v>
+        <x:v>弦乐器</x:v>
       </x:c>
       <x:c r="E13" s="40" t="str">
         <x:v>古典</x:v>
@@ -2830,10 +2830,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="X13" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"global","filter":{"tag1":["提琴声部"]},"cap":5,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"global","filter":{"category":["弦乐器"]},"cap":5,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y13" s="44" t="str">
-        <x:v>使背包中的其他提琴声部道具各增加[3／4／5／6／8]%表演值，最多5件</x:v>
+        <x:v>使背包中的其他弦乐器道具各增加[3／4／5／6／8]%表演值，最多5件</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
@@ -2847,7 +2847,7 @@
         <x:v>弦乐器</x:v>
       </x:c>
       <x:c r="D14" s="40" t="str">
-        <x:v>提琴声部</x:v>
+        <x:v>弦乐器</x:v>
       </x:c>
       <x:c r="E14" s="40" t="str">
         <x:v>古典</x:v>
@@ -2908,10 +2908,10 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="X14" s="40" t="str">
-        <x:v>{"type":"count","scope":"global","filter":{"tag1":["提琴声部"]},"cap":4,"excludeSource":true,"excludeAdjacent":true,"directions":[],"valueMode":"percent","recipient":"self"}</x:v>
+        <x:v>{"type":"count","scope":"global","filter":{"category":["弦乐器"]},"cap":4,"excludeSource":true,"excludeAdjacent":true,"directions":[],"valueMode":"percent","recipient":"self"}</x:v>
       </x:c>
       <x:c r="Y14" s="44" t="str">
-        <x:v>背包中每有1件与自身不相邻的提琴声部道具，自身表演值增加[2／3／4／5／6]%，最多4件</x:v>
+        <x:v>背包中每有1件与自身不相邻的弦乐器道具，自身表演值增加[2／3／4／5／6]%，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
@@ -2925,7 +2925,7 @@
         <x:v>弦乐器</x:v>
       </x:c>
       <x:c r="D15" s="40" t="str">
-        <x:v>提琴声部</x:v>
+        <x:v>弦乐器</x:v>
       </x:c>
       <x:c r="E15" s="40" t="str">
         <x:v>古典</x:v>
@@ -2986,10 +2986,10 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="X15" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["提琴声部"]},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"category":["弦乐器"]},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y15" s="44" t="str">
-        <x:v>使相邻的其他提琴声部道具各增加[4／5／7／9／11]表演值，最多3件</x:v>
+        <x:v>使相邻的其他弦乐器道具各增加[4／5／7／9／11]表演值，最多3件</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
@@ -3003,7 +3003,7 @@
         <x:v>弦乐器</x:v>
       </x:c>
       <x:c r="D16" s="40" t="str">
-        <x:v>提琴声部</x:v>
+        <x:v>弦乐器</x:v>
       </x:c>
       <x:c r="E16" s="40" t="str">
         <x:v>古典</x:v>
@@ -3064,10 +3064,10 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="X16" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["提琴声部"]},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"category":["弦乐器"]},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y16" s="44" t="str">
-        <x:v>使相邻的其他提琴声部道具各增加[5／7／9／11／14]表演值，最多3件</x:v>
+        <x:v>使相邻的其他弦乐器道具各增加[5／7／9／11／14]表演值，最多3件</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
@@ -3081,7 +3081,7 @@
         <x:v>弦乐器</x:v>
       </x:c>
       <x:c r="D17" s="40" t="str">
-        <x:v>提琴声部</x:v>
+        <x:v>弦乐器</x:v>
       </x:c>
       <x:c r="E17" s="40" t="str">
         <x:v>现代</x:v>
@@ -3142,10 +3142,10 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="X17" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["现代"]},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"category":["键盘乐器","弦乐器","管乐器","打击乐器"]},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y17" s="44" t="str">
-        <x:v>使相邻的现代乐器标签道具各增加[4／5／7／9／11]表演值，最多3件，不计自身</x:v>
+        <x:v>使相邻的乐器道具各增加[4／5／7／9／11]表演值，最多3件，不计自身</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
@@ -3159,7 +3159,7 @@
         <x:v>弦乐器</x:v>
       </x:c>
       <x:c r="D18" s="40" t="str">
-        <x:v>提琴声部</x:v>
+        <x:v>弦乐器</x:v>
       </x:c>
       <x:c r="E18" s="40" t="str">
         <x:v>古典</x:v>
@@ -3220,10 +3220,10 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="X18" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["提琴声部"]},"cap":1,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"category":["弦乐器"]},"cap":1,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y18" s="44" t="str">
-        <x:v>使相邻的1件其他提琴声部道具增加[7／9／12／14／18]表演值</x:v>
+        <x:v>使相邻的1件其他弦乐器道具增加[7／9／12／14／18]表演值</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
@@ -3237,7 +3237,7 @@
         <x:v>弦乐器</x:v>
       </x:c>
       <x:c r="D19" s="40" t="str">
-        <x:v>拨弦声部</x:v>
+        <x:v>弦乐器</x:v>
       </x:c>
       <x:c r="E19" s="40" t="str">
         <x:v>现代</x:v>
@@ -3298,10 +3298,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="X19" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["拨弦声部"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"category":["弦乐器"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y19" s="44" t="str">
-        <x:v>使相邻的拨弦声部道具各增加[4／5／6／8／10]表演值，最多2件，不计自身</x:v>
+        <x:v>使相邻的弦乐器道具各增加[4／5／6／8／10]表演值，最多2件，不计自身</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
@@ -3315,7 +3315,7 @@
         <x:v>弦乐器</x:v>
       </x:c>
       <x:c r="D20" s="40" t="str">
-        <x:v>拨弦声部</x:v>
+        <x:v>弦乐器</x:v>
       </x:c>
       <x:c r="E20" s="40" t="str">
         <x:v>现代</x:v>
@@ -3376,10 +3376,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="X20" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"global","filter":{"tag1":["拨弦声部"]},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"global","filter":{"category":["弦乐器"]},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y20" s="44" t="str">
-        <x:v>使背包中的其他拨弦声部道具各增加[3／4／5／6／8]表演值，最多3件</x:v>
+        <x:v>使背包中的其他弦乐器道具各增加[3／4／5／6／8]表演值，最多3件</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="42" customHeight="1">
@@ -3393,7 +3393,7 @@
         <x:v>弦乐器</x:v>
       </x:c>
       <x:c r="D21" s="40" t="str">
-        <x:v>提琴声部</x:v>
+        <x:v>弦乐器</x:v>
       </x:c>
       <x:c r="E21" s="40" t="str">
         <x:v>古典</x:v>
@@ -3454,10 +3454,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="X21" s="40" t="str">
-        <x:v>{"type":"condition","clauses":[{"scope":"adjacent","filter":{"tag1":["提琴声部"]},"min":null,"max":0,"cap":null,"excludeSource":true,"directions":[]}],"valueMode":"absolute","recipient":"self"}</x:v>
+        <x:v>{"type":"condition","clauses":[{"scope":"adjacent","filter":{"category":["弦乐器"]},"min":null,"max":0,"cap":null,"excludeSource":true,"directions":[]}],"valueMode":"absolute","recipient":"self"}</x:v>
       </x:c>
       <x:c r="Y21" s="44" t="str">
-        <x:v>与其他提琴声部道具均不相邻时，自身增加[10／13／17／21／25]表演值</x:v>
+        <x:v>与其他弦乐器道具均不相邻时，自身增加[10／13／17／21／25]表演值</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
@@ -3471,7 +3471,7 @@
         <x:v>管乐器</x:v>
       </x:c>
       <x:c r="D22" s="40" t="str">
-        <x:v>铜管声部</x:v>
+        <x:v>管乐器</x:v>
       </x:c>
       <x:c r="E22" s="40" t="str">
         <x:v>古典</x:v>
@@ -3532,10 +3532,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="X22" s="40" t="str">
-        <x:v>{"type":"balance","a":{"scope":"global","filter":{"tag1":["木管声部"]}},"b":{"scope":"global","filter":{"tag1":["铜管声部"]}},"minEach":2,"maxDiff":1,"capEach":4,"excludeSource":true,"valueMode":"percent","recipient":"self"}</x:v>
+        <x:v>{"type":"condition","clauses":[{"scope":"global","filter":{"category":["管乐器"]},"min":4,"max":null,"cap":null,"excludeSource":true,"directions":[]}],"valueMode":"percent","recipient":"self"}</x:v>
       </x:c>
       <x:c r="Y22" s="44" t="str">
-        <x:v>背包中木管声部与铜管声部数量差不超过1且各至少2件时，自身表演值增加[10／13／16／20／25]%</x:v>
+        <x:v>背包中至少有4件其他管乐器时，自身表演值增加[10／13／16／20／25]%</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
@@ -3549,7 +3549,7 @@
         <x:v>管乐器</x:v>
       </x:c>
       <x:c r="D23" s="40" t="str">
-        <x:v>木管声部</x:v>
+        <x:v>管乐器</x:v>
       </x:c>
       <x:c r="E23" s="40" t="str">
         <x:v>古典</x:v>
@@ -3610,10 +3610,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="X23" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["木管声部"]},"cap":4,"excludeSource":true,"directions":["up","down"],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"category":["管乐器"]},"cap":4,"excludeSource":true,"directions":["up","down"],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y23" s="44" t="str">
-        <x:v>使上方和下方的其他木管声部道具各增加[3／4／5／6／8]%表演值，最多4件</x:v>
+        <x:v>使上方和下方的其他管乐器道具各增加[3／4／5／6／8]%表演值，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
@@ -3627,7 +3627,7 @@
         <x:v>管乐器</x:v>
       </x:c>
       <x:c r="D24" s="40" t="str">
-        <x:v>铜管声部</x:v>
+        <x:v>管乐器</x:v>
       </x:c>
       <x:c r="E24" s="40" t="str">
         <x:v>古典</x:v>
@@ -3688,10 +3688,10 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="X24" s="40" t="str">
-        <x:v>{"type":"groupBuff","clauses":[{"scope":"direction","filter":{"tag1":["铜管声部"]},"min":1,"max":null,"cap":null,"excludeSource":true,"directions":["left"]},{"scope":"direction","filter":{"tag1":["铜管声部"]},"min":1,"max":null,"cap":null,"excludeSource":true,"directions":["right"]}],"recipients":{"scope":"direction","directions":["left","right"],"filter":{"tag1":["铜管声部"]},"cap":4,"includeSource":false},"valueMode":"percent"}</x:v>
+        <x:v>{"type":"groupBuff","clauses":[{"scope":"direction","filter":{"category":["管乐器"]},"min":1,"max":null,"cap":null,"excludeSource":true,"directions":["left"]},{"scope":"direction","filter":{"category":["管乐器"]},"min":1,"max":null,"cap":null,"excludeSource":true,"directions":["right"]}],"recipients":{"scope":"direction","directions":["left","right"],"filter":{"category":["管乐器"]},"cap":4,"includeSource":false},"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y24" s="44" t="str">
-        <x:v>左侧和右侧各至少有1件其他铜管声部道具时，使两侧符合条件的道具各增加[5／6／8／10／12]%表演值，最多4件</x:v>
+        <x:v>左侧和右侧各至少有1件其他管乐器道具时，使两侧符合条件的道具各增加[5／6／8／10／12]%表演值，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
@@ -3705,7 +3705,7 @@
         <x:v>管乐器</x:v>
       </x:c>
       <x:c r="D25" s="40" t="str">
-        <x:v>木管声部</x:v>
+        <x:v>管乐器</x:v>
       </x:c>
       <x:c r="E25" s="40" t="str">
         <x:v>古典</x:v>
@@ -3766,10 +3766,10 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="X25" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["木管声部"]},"cap":3,"excludeSource":true,"directions":["up"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"category":["管乐器"]},"cap":3,"excludeSource":true,"directions":["up"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y25" s="44" t="str">
-        <x:v>使上方的其他木管声部道具各增加[5／6／8／10／12]表演值，最多3件</x:v>
+        <x:v>使上方的其他管乐器道具各增加[5／6／8／10／12]表演值，最多3件</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="42" customHeight="1">
@@ -3783,7 +3783,7 @@
         <x:v>管乐器</x:v>
       </x:c>
       <x:c r="D26" s="40" t="str">
-        <x:v>铜管声部</x:v>
+        <x:v>管乐器</x:v>
       </x:c>
       <x:c r="E26" s="40" t="str">
         <x:v>现代</x:v>
@@ -3844,10 +3844,10 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="X26" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["铜管声部"]},"cap":3,"excludeSource":true,"directions":["right"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"category":["管乐器"]},"cap":3,"excludeSource":true,"directions":["right"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y26" s="44" t="str">
-        <x:v>使右侧的其他铜管声部道具各增加[5／6／8／10／12]表演值，最多3件</x:v>
+        <x:v>使右侧的其他管乐器道具各增加[5／6／8／10／12]表演值，最多3件</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="42" customHeight="1">
@@ -3861,7 +3861,7 @@
         <x:v>管乐器</x:v>
       </x:c>
       <x:c r="D27" s="40" t="str">
-        <x:v>木管声部</x:v>
+        <x:v>管乐器</x:v>
       </x:c>
       <x:c r="E27" s="40" t="str">
         <x:v>现代</x:v>
@@ -3922,10 +3922,10 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="X27" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"global","filter":{"tag1":["木管声部"]},"cap":4,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"global","filter":{"category":["管乐器"]},"cap":4,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y27" s="44" t="str">
-        <x:v>使背包中的其他木管声部道具各增加[4／5／7／9／11]表演值，最多4件</x:v>
+        <x:v>使背包中的其他管乐器道具各增加[4／5／7／9／11]表演值，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="42" customHeight="1">
@@ -3939,7 +3939,7 @@
         <x:v>管乐器</x:v>
       </x:c>
       <x:c r="D28" s="40" t="str">
-        <x:v>铜管声部</x:v>
+        <x:v>管乐器</x:v>
       </x:c>
       <x:c r="E28" s="40" t="str">
         <x:v>现代</x:v>
@@ -4000,10 +4000,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="X28" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["铜管声部"]},"cap":2,"excludeSource":true,"directions":["left"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"category":["管乐器"]},"cap":2,"excludeSource":true,"directions":["left"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y28" s="44" t="str">
-        <x:v>使左侧的其他铜管声部道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
+        <x:v>使左侧的其他管乐器道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
@@ -4017,7 +4017,7 @@
         <x:v>管乐器</x:v>
       </x:c>
       <x:c r="D29" s="40" t="str">
-        <x:v>木管声部</x:v>
+        <x:v>管乐器</x:v>
       </x:c>
       <x:c r="E29" s="40" t="str">
         <x:v>古典</x:v>
@@ -4078,10 +4078,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="X29" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["木管声部"]},"cap":2,"excludeSource":true,"directions":["down"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"category":["管乐器"]},"cap":2,"excludeSource":true,"directions":["down"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y29" s="44" t="str">
-        <x:v>使下方的其他木管声部道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
+        <x:v>使下方的其他管乐器道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="42" customHeight="1">
@@ -4095,7 +4095,7 @@
         <x:v>管乐器</x:v>
       </x:c>
       <x:c r="D30" s="40" t="str">
-        <x:v>铜管声部</x:v>
+        <x:v>管乐器</x:v>
       </x:c>
       <x:c r="E30" s="40" t="str">
         <x:v>现代</x:v>
@@ -4156,10 +4156,10 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="X30" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["铜管声部"]},"cap":1,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"category":["管乐器"]},"cap":1,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y30" s="44" t="str">
-        <x:v>使相邻的1件其他铜管声部道具增加[7／9／12／14／18]表演值</x:v>
+        <x:v>使相邻的1件其他管乐器道具增加[7／9／12／14／18]表演值</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
@@ -4173,7 +4173,7 @@
         <x:v>管乐器</x:v>
       </x:c>
       <x:c r="D31" s="40" t="str">
-        <x:v>木管声部</x:v>
+        <x:v>管乐器</x:v>
       </x:c>
       <x:c r="E31" s="40" t="str">
         <x:v>古典</x:v>
@@ -4234,10 +4234,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="X31" s="40" t="str">
-        <x:v>{"type":"condition","clauses":[{"scope":"adjacent","filter":{"tag1":["木管声部"]},"min":null,"max":0,"cap":null,"excludeSource":true,"directions":[]}],"valueMode":"absolute","recipient":"self"}</x:v>
+        <x:v>{"type":"condition","clauses":[{"scope":"adjacent","filter":{"category":["管乐器"]},"min":null,"max":0,"cap":null,"excludeSource":true,"directions":[]}],"valueMode":"absolute","recipient":"self"}</x:v>
       </x:c>
       <x:c r="Y31" s="44" t="str">
-        <x:v>与其他木管声部道具均不相邻时，自身增加[10／13／17／21／25]表演值</x:v>
+        <x:v>与其他管乐器道具均不相邻时，自身增加[10／13／17／21／25]表演值</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="42" customHeight="1">
@@ -4251,7 +4251,7 @@
         <x:v>打击乐器</x:v>
       </x:c>
       <x:c r="D32" s="40" t="str">
-        <x:v>管弦打击</x:v>
+        <x:v>打击乐器</x:v>
       </x:c>
       <x:c r="E32" s="40" t="str">
         <x:v>古典</x:v>
@@ -4312,10 +4312,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="X32" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["管弦打击"]},"cap":4,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"category":["打击乐器"]},"cap":4,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y32" s="44" t="str">
-        <x:v>使相邻的其他管弦打击道具各增加[4／5／6／8／10]%表演值，最多4件</x:v>
+        <x:v>使相邻的其他打击乐器道具各增加[4／5／6／8／10]%表演值，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
@@ -4329,7 +4329,7 @@
         <x:v>打击乐器</x:v>
       </x:c>
       <x:c r="D33" s="40" t="str">
-        <x:v>管弦打击</x:v>
+        <x:v>打击乐器</x:v>
       </x:c>
       <x:c r="E33" s="40" t="str">
         <x:v>古典</x:v>
@@ -4390,10 +4390,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="X33" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["管弦打击"]},"cap":4,"excludeSource":true,"directions":["up","down"],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"category":["打击乐器"]},"cap":4,"excludeSource":true,"directions":["up","down"],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y33" s="44" t="str">
-        <x:v>使上方和下方的其他管弦打击道具各增加[3／4／5／6／8]%表演值，最多4件</x:v>
+        <x:v>使上方和下方的其他打击乐器道具各增加[3／4／5／6／8]%表演值，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="42" customHeight="1">
@@ -4407,7 +4407,7 @@
         <x:v>打击乐器</x:v>
       </x:c>
       <x:c r="D34" s="40" t="str">
-        <x:v>节奏打击</x:v>
+        <x:v>打击乐器</x:v>
       </x:c>
       <x:c r="E34" s="40" t="str">
         <x:v>现代</x:v>
@@ -4468,10 +4468,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="X34" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["节奏打击"]},"cap":4,"excludeSource":true,"directions":["left","right"],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"category":["打击乐器"]},"cap":4,"excludeSource":true,"directions":["left","right"],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y34" s="44" t="str">
-        <x:v>使左侧和右侧的其他节奏打击道具各增加[3／4／5／6／8]%表演值，最多4件</x:v>
+        <x:v>使左侧和右侧的其他打击乐器道具各增加[3／4／5／6／8]%表演值，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="42" customHeight="1">
@@ -4485,7 +4485,7 @@
         <x:v>打击乐器</x:v>
       </x:c>
       <x:c r="D35" s="40" t="str">
-        <x:v>管弦打击</x:v>
+        <x:v>打击乐器</x:v>
       </x:c>
       <x:c r="E35" s="40" t="str">
         <x:v>古典</x:v>
@@ -4546,10 +4546,10 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="X35" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["管弦打击"]},"cap":3,"excludeSource":true,"directions":["down"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"category":["打击乐器"]},"cap":3,"excludeSource":true,"directions":["down"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y35" s="44" t="str">
-        <x:v>使下方的其他管弦打击道具各增加[5／7／9／11／14]表演值，最多3件</x:v>
+        <x:v>使下方的其他打击乐器道具各增加[5／7／9／11／14]表演值，最多3件</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="42" customHeight="1">
@@ -4563,7 +4563,7 @@
         <x:v>打击乐器</x:v>
       </x:c>
       <x:c r="D36" s="40" t="str">
-        <x:v>管弦打击</x:v>
+        <x:v>打击乐器</x:v>
       </x:c>
       <x:c r="E36" s="40" t="str">
         <x:v>古典</x:v>
@@ -4624,10 +4624,10 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="X36" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["管弦打击"]},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"category":["打击乐器"]},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y36" s="44" t="str">
-        <x:v>使相邻的其他管弦打击道具各增加[5／6／8／10／12]表演值，最多3件</x:v>
+        <x:v>使相邻的其他打击乐器道具各增加[5／6／8／10／12]表演值，最多3件</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="42" customHeight="1">
@@ -4641,7 +4641,7 @@
         <x:v>打击乐器</x:v>
       </x:c>
       <x:c r="D37" s="40" t="str">
-        <x:v>节奏打击</x:v>
+        <x:v>打击乐器</x:v>
       </x:c>
       <x:c r="E37" s="40" t="str">
         <x:v>现代</x:v>
@@ -4702,10 +4702,10 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="X37" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["节奏打击"]},"cap":3,"excludeSource":true,"directions":["left"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"category":["打击乐器"]},"cap":3,"excludeSource":true,"directions":["left"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y37" s="44" t="str">
-        <x:v>使左侧的其他节奏打击道具各增加[5／6／8／10／12]表演值，最多3件</x:v>
+        <x:v>使左侧的其他打击乐器道具各增加[5／6／8／10／12]表演值，最多3件</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="42" customHeight="1">
@@ -4719,7 +4719,7 @@
         <x:v>打击乐器</x:v>
       </x:c>
       <x:c r="D38" s="40" t="str">
-        <x:v>管弦打击</x:v>
+        <x:v>打击乐器</x:v>
       </x:c>
       <x:c r="E38" s="40" t="str">
         <x:v>现代</x:v>
@@ -4780,10 +4780,10 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="X38" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["管弦打击"]},"cap":1,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"category":["打击乐器"]},"cap":1,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y38" s="44" t="str">
-        <x:v>使相邻的1件其他管弦打击道具增加[7／9／12／14／18]表演值</x:v>
+        <x:v>使相邻的1件其他打击乐器道具增加[7／9／12／14／18]表演值</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="42" customHeight="1">
@@ -4797,7 +4797,7 @@
         <x:v>打击乐器</x:v>
       </x:c>
       <x:c r="D39" s="40" t="str">
-        <x:v>节奏打击</x:v>
+        <x:v>打击乐器</x:v>
       </x:c>
       <x:c r="E39" s="40" t="str">
         <x:v>现代</x:v>
@@ -4858,10 +4858,10 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="X39" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["节奏打击"]},"cap":1,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"category":["打击乐器"]},"cap":1,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y39" s="44" t="str">
-        <x:v>使相邻的1件其他节奏打击道具增加[7／9／12／14／18]表演值</x:v>
+        <x:v>使相邻的1件其他打击乐器道具增加[7／9／12／14／18]表演值</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="42" customHeight="1">
@@ -4875,7 +4875,7 @@
         <x:v>打击乐器</x:v>
       </x:c>
       <x:c r="D40" s="40" t="str">
-        <x:v>管弦打击</x:v>
+        <x:v>打击乐器</x:v>
       </x:c>
       <x:c r="E40" s="40" t="str">
         <x:v>古典</x:v>
@@ -4936,10 +4936,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="X40" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["管弦打击","节奏打击"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"category":["打击乐器"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y40" s="44" t="str">
-        <x:v>使相邻的其他管弦打击或节奏打击道具各增加[3／4／5／6／8]表演值，最多2件</x:v>
+        <x:v>使相邻的其他打击乐器道具各增加[3／4／5／6／8]表演值，最多2件</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="42" customHeight="1">
@@ -4953,7 +4953,7 @@
         <x:v>打击乐器</x:v>
       </x:c>
       <x:c r="D41" s="40" t="str">
-        <x:v>节奏打击</x:v>
+        <x:v>打击乐器</x:v>
       </x:c>
       <x:c r="E41" s="40" t="str">
         <x:v>现代</x:v>
@@ -5014,10 +5014,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="X41" s="40" t="str">
-        <x:v>{"type":"condition","clauses":[{"scope":"adjacent","filter":{"tag1":["节奏打击"]},"min":null,"max":0,"cap":null,"excludeSource":true,"directions":[]}],"valueMode":"absolute","recipient":"self"}</x:v>
+        <x:v>{"type":"condition","clauses":[{"scope":"adjacent","filter":{"category":["打击乐器"]},"min":null,"max":0,"cap":null,"excludeSource":true,"directions":[]}],"valueMode":"absolute","recipient":"self"}</x:v>
       </x:c>
       <x:c r="Y41" s="44" t="str">
-        <x:v>与其他节奏打击道具均不相邻时，自身增加[10／13／17／21／25]表演值</x:v>
+        <x:v>与其他打击乐器道具均不相邻时，自身增加[10／13／17／21／25]表演值</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="42" customHeight="1">
@@ -5031,7 +5031,7 @@
         <x:v>服装</x:v>
       </x:c>
       <x:c r="D42" s="40" t="str">
-        <x:v>芭蕾服装</x:v>
+        <x:v>服装</x:v>
       </x:c>
       <x:c r="E42" s="40" t="str">
         <x:v>古典</x:v>
@@ -5092,10 +5092,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="X42" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"global","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["古典"]},"cap":6,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"global","filter":{"category":["键盘乐器","弦乐器","管乐器","打击乐器"]},"cap":6,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y42" s="44" t="str">
-        <x:v>使背包中的古典乐器标签道具各增加[3／4／5／6／8]%表演值，最多6件</x:v>
+        <x:v>使背包中的乐器道具各增加[3／4／5／6／8]%表演值，最多6件</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="42" customHeight="1">
@@ -5109,7 +5109,7 @@
         <x:v>服装</x:v>
       </x:c>
       <x:c r="D43" s="40" t="str">
-        <x:v>芭蕾服装</x:v>
+        <x:v>服装</x:v>
       </x:c>
       <x:c r="E43" s="40" t="str">
         <x:v>古典</x:v>
@@ -5170,10 +5170,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="X43" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["提琴声部"]},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"category":["弦乐器"]},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y43" s="44" t="str">
-        <x:v>使相邻的提琴声部道具各增加[4／5／6／8／10]%表演值，最多3件</x:v>
+        <x:v>使相邻的弦乐器道具各增加[4／5／6／8／10]%表演值，最多3件</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="42" customHeight="1">
@@ -5187,7 +5187,7 @@
         <x:v>服装</x:v>
       </x:c>
       <x:c r="D44" s="40" t="str">
-        <x:v>歌剧服装</x:v>
+        <x:v>服装</x:v>
       </x:c>
       <x:c r="E44" s="40" t="str">
         <x:v>古典</x:v>
@@ -5248,10 +5248,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="X44" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["古典"]},"cap":4,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"category":["键盘乐器","弦乐器","管乐器","打击乐器"]},"cap":4,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y44" s="44" t="str">
-        <x:v>使相邻的古典乐器标签道具各增加[3／4／5／6／8]%表演值，最多4件</x:v>
+        <x:v>使相邻的乐器道具各增加[3／4／5／6／8]%表演值，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="42" customHeight="1">
@@ -5265,7 +5265,7 @@
         <x:v>服装</x:v>
       </x:c>
       <x:c r="D45" s="40" t="str">
-        <x:v>爵士服装</x:v>
+        <x:v>服装</x:v>
       </x:c>
       <x:c r="E45" s="40" t="str">
         <x:v>现代</x:v>
@@ -5326,10 +5326,10 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="X45" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["现代"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"category":["键盘乐器","弦乐器","管乐器","打击乐器"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y45" s="44" t="str">
-        <x:v>使相邻的现代乐器标签道具各增加[7／9／12／14／18]表演值，最多2件</x:v>
+        <x:v>使相邻的乐器道具各增加[7／9／12／14／18]表演值，最多2件</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="42" customHeight="1">
@@ -5343,7 +5343,7 @@
         <x:v>服装</x:v>
       </x:c>
       <x:c r="D46" s="40" t="str">
-        <x:v>歌剧服装</x:v>
+        <x:v>服装</x:v>
       </x:c>
       <x:c r="E46" s="40" t="str">
         <x:v>古典</x:v>
@@ -5404,10 +5404,10 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="X46" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"global","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["古典"]},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"global","filter":{"category":["键盘乐器","弦乐器","管乐器","打击乐器"]},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y46" s="44" t="str">
-        <x:v>使背包中的古典乐器标签道具各增加[5／6／8／10／12]表演值，最多3件</x:v>
+        <x:v>使背包中的乐器道具各增加[5／6／8／10／12]表演值，最多3件</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="42" customHeight="1">
@@ -5421,7 +5421,7 @@
         <x:v>服装</x:v>
       </x:c>
       <x:c r="D47" s="40" t="str">
-        <x:v>爵士服装</x:v>
+        <x:v>服装</x:v>
       </x:c>
       <x:c r="E47" s="40" t="str">
         <x:v>现代</x:v>
@@ -5482,10 +5482,10 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="X47" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["现代"]},"cap":3,"excludeSource":true,"directions":["left","right"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"category":["键盘乐器","弦乐器","管乐器","打击乐器"]},"cap":3,"excludeSource":true,"directions":["left","right"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y47" s="44" t="str">
-        <x:v>使左侧和右侧的现代乐器标签道具各增加[5／6／8／10／12]表演值，最多3件</x:v>
+        <x:v>使左侧和右侧的乐器道具各增加[5／6／8／10／12]表演值，最多3件</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="42" customHeight="1">
@@ -5499,7 +5499,7 @@
         <x:v>服装</x:v>
       </x:c>
       <x:c r="D48" s="40" t="str">
-        <x:v>芭蕾服装</x:v>
+        <x:v>服装</x:v>
       </x:c>
       <x:c r="E48" s="40" t="str">
         <x:v>古典</x:v>
@@ -5560,10 +5560,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="X48" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["提琴声部"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"category":["弦乐器"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y48" s="44" t="str">
-        <x:v>使相邻的提琴声部道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
+        <x:v>使相邻的弦乐器道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="42" customHeight="1">
@@ -5577,7 +5577,7 @@
         <x:v>服装</x:v>
       </x:c>
       <x:c r="D49" s="40" t="str">
-        <x:v>芭蕾服装</x:v>
+        <x:v>服装</x:v>
       </x:c>
       <x:c r="E49" s="40" t="str">
         <x:v>古典</x:v>
@@ -5638,10 +5638,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="X49" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["提琴声部"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"category":["弦乐器"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y49" s="44" t="str">
-        <x:v>使相邻的提琴声部道具各增加[3／4／5／6／8]表演值，最多2件</x:v>
+        <x:v>使相邻的弦乐器道具各增加[3／4／5／6／8]表演值，最多2件</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="42" customHeight="1">
@@ -5655,7 +5655,7 @@
         <x:v>服装</x:v>
       </x:c>
       <x:c r="D50" s="40" t="str">
-        <x:v>歌剧服装</x:v>
+        <x:v>服装</x:v>
       </x:c>
       <x:c r="E50" s="40" t="str">
         <x:v>古典</x:v>
@@ -5716,10 +5716,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="X50" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"global","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["古典"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"global","filter":{"category":["键盘乐器","弦乐器","管乐器","打击乐器"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y50" s="44" t="str">
-        <x:v>使背包中的古典乐器标签道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
+        <x:v>使背包中的乐器道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="42" customHeight="1">
@@ -5733,7 +5733,7 @@
         <x:v>服装</x:v>
       </x:c>
       <x:c r="D51" s="40" t="str">
-        <x:v>爵士服装</x:v>
+        <x:v>服装</x:v>
       </x:c>
       <x:c r="E51" s="40" t="str">
         <x:v>现代</x:v>
@@ -5794,10 +5794,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="X51" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["现代"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"category":["键盘乐器","弦乐器","管乐器","打击乐器"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y51" s="44" t="str">
-        <x:v>使相邻的现代乐器标签道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
+        <x:v>使相邻的乐器道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="42" customHeight="1">
@@ -5811,7 +5811,7 @@
         <x:v>舞台装饰</x:v>
       </x:c>
       <x:c r="D52" s="40" t="str">
-        <x:v>布景</x:v>
+        <x:v>舞台装饰</x:v>
       </x:c>
       <x:c r="E52" s="40" t="str">
         <x:v>古典</x:v>
@@ -5872,10 +5872,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="X52" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"global","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["古典"]},"cap":6,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"global","filter":{"category":["键盘乐器","弦乐器","管乐器","打击乐器"]},"cap":6,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y52" s="44" t="str">
-        <x:v>使背包中的古典乐器标签道具各增加[4／5／6／8／10]%表演值，最多6件</x:v>
+        <x:v>使背包中的乐器道具各增加[4／5／6／8／10]%表演值，最多6件</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="42" customHeight="1">
@@ -5889,7 +5889,7 @@
         <x:v>舞台装饰</x:v>
       </x:c>
       <x:c r="D53" s="40" t="str">
-        <x:v>灯光</x:v>
+        <x:v>舞台装饰</x:v>
       </x:c>
       <x:c r="E53" s="40" t="str">
         <x:v>古典</x:v>
@@ -5950,10 +5950,10 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="X53" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"]},"cap":4,"excludeSource":true,"directions":["left","right"],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"category":["键盘乐器","弦乐器","管乐器","打击乐器"]},"cap":4,"excludeSource":true,"directions":["left","right"],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y53" s="44" t="str">
-        <x:v>使左侧和右侧的乐器标签道具各增加[3／4／5／6／8]%表演值，最多4件</x:v>
+        <x:v>使左侧和右侧的乐器道具各增加[3／4／5／6／8]%表演值，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="42" customHeight="1">
@@ -5967,7 +5967,7 @@
         <x:v>舞台装饰</x:v>
       </x:c>
       <x:c r="D54" s="40" t="str">
-        <x:v>声场</x:v>
+        <x:v>舞台装饰</x:v>
       </x:c>
       <x:c r="E54" s="40" t="str">
         <x:v>现代</x:v>
@@ -6028,10 +6028,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="X54" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"global","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"minArea":4},"cap":4,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"global","filter":{"minArea":4,"category":["键盘乐器","弦乐器","管乐器","打击乐器"]},"cap":4,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"percent"}</x:v>
       </x:c>
       <x:c r="Y54" s="44" t="str">
-        <x:v>使背包中占用4格及以上的乐器标签道具各增加[4／5／6／8／10]%表演值，最多4件</x:v>
+        <x:v>使背包中占用4格及以上的乐器道具各增加[4／5／6／8／10]%表演值，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="42" customHeight="1">
@@ -6045,7 +6045,7 @@
         <x:v>舞台装饰</x:v>
       </x:c>
       <x:c r="D55" s="40" t="str">
-        <x:v>灯光</x:v>
+        <x:v>舞台装饰</x:v>
       </x:c>
       <x:c r="E55" s="40" t="str">
         <x:v>古典</x:v>
@@ -6106,10 +6106,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="X55" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"]},"cap":4,"excludeSource":true,"directions":["up"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"category":["键盘乐器","弦乐器","管乐器","打击乐器"]},"cap":4,"excludeSource":true,"directions":["up"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y55" s="44" t="str">
-        <x:v>使上方的乐器标签道具各增加[4／5／6／8／10]表演值，最多4件</x:v>
+        <x:v>使上方的乐器道具各增加[4／5／6／8／10]表演值，最多4件</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="42" customHeight="1">
@@ -6123,7 +6123,7 @@
         <x:v>舞台装饰</x:v>
       </x:c>
       <x:c r="D56" s="40" t="str">
-        <x:v>布景</x:v>
+        <x:v>舞台装饰</x:v>
       </x:c>
       <x:c r="E56" s="40" t="str">
         <x:v>古典</x:v>
@@ -6184,10 +6184,10 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="X56" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"direction","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["古典"]},"cap":3,"excludeSource":true,"directions":["left","right"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"direction","filter":{"category":["键盘乐器","弦乐器","管乐器","打击乐器"]},"cap":3,"excludeSource":true,"directions":["left","right"],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y56" s="44" t="str">
-        <x:v>使左侧和右侧的古典乐器标签道具各增加[5／6／8／10／12]表演值，最多3件</x:v>
+        <x:v>使左侧和右侧的乐器道具各增加[5／6／8／10／12]表演值，最多3件</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="42" customHeight="1">
@@ -6201,7 +6201,7 @@
         <x:v>舞台装饰</x:v>
       </x:c>
       <x:c r="D57" s="40" t="str">
-        <x:v>声场</x:v>
+        <x:v>舞台装饰</x:v>
       </x:c>
       <x:c r="E57" s="40" t="str">
         <x:v>现代</x:v>
@@ -6262,10 +6262,10 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="X57" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"global","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"]},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"global","filter":{"category":["键盘乐器","弦乐器","管乐器","打击乐器"]},"cap":3,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y57" s="44" t="str">
-        <x:v>使背包中的乐器标签道具各增加[5／6／8／10／12]表演值，最多3件</x:v>
+        <x:v>使背包中的乐器道具各增加[5／6／8／10／12]表演值，最多3件</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="42" customHeight="1">
@@ -6279,7 +6279,7 @@
         <x:v>舞台装饰</x:v>
       </x:c>
       <x:c r="D58" s="40" t="str">
-        <x:v>灯光</x:v>
+        <x:v>舞台装饰</x:v>
       </x:c>
       <x:c r="E58" s="40" t="str">
         <x:v>现代</x:v>
@@ -6340,10 +6340,10 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="X58" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["现代"]},"cap":1,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"category":["键盘乐器","弦乐器","管乐器","打击乐器"]},"cap":1,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y58" s="44" t="str">
-        <x:v>使相邻的1件现代乐器标签道具增加[8／10／13／16／20]表演值</x:v>
+        <x:v>使相邻的1件乐器道具增加[8／10／13／16／20]表演值</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="42" customHeight="1">
@@ -6357,7 +6357,7 @@
         <x:v>舞台装饰</x:v>
       </x:c>
       <x:c r="D59" s="40" t="str">
-        <x:v>布景</x:v>
+        <x:v>舞台装饰</x:v>
       </x:c>
       <x:c r="E59" s="40" t="str">
         <x:v>古典</x:v>
@@ -6418,10 +6418,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="X59" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"],"tag2":["古典"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"category":["键盘乐器","弦乐器","管乐器","打击乐器"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y59" s="44" t="str">
-        <x:v>使相邻的古典乐器标签道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
+        <x:v>使相邻的乐器道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="42" customHeight="1">
@@ -6435,7 +6435,7 @@
         <x:v>舞台装饰</x:v>
       </x:c>
       <x:c r="D60" s="40" t="str">
-        <x:v>灯光</x:v>
+        <x:v>舞台装饰</x:v>
       </x:c>
       <x:c r="E60" s="40" t="str">
         <x:v>现代</x:v>
@@ -6496,10 +6496,10 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="X60" s="40" t="str">
-        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"]},"cap":1,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"adjacent","filter":{"category":["键盘乐器","弦乐器","管乐器","打击乐器"]},"cap":1,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y60" s="44" t="str">
-        <x:v>使相邻的1件乐器标签道具增加[8／10／13／16／20]表演值</x:v>
+        <x:v>使相邻的1件乐器道具增加[8／10／13／16／20]表演值</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="42" customHeight="1">
@@ -6513,7 +6513,7 @@
         <x:v>舞台装饰</x:v>
       </x:c>
       <x:c r="D61" s="42" t="str">
-        <x:v>声场</x:v>
+        <x:v>舞台装饰</x:v>
       </x:c>
       <x:c r="E61" s="42" t="str">
         <x:v>现代</x:v>
@@ -6574,10 +6574,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="X61" s="42" t="str">
-        <x:v>{"type":"targetBuff","scope":"global","filter":{"tag1":["钢琴键盘","管风琴键盘","提琴声部","拨弦声部","木管声部","铜管声部","管弦打击","节奏打击"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
+        <x:v>{"type":"targetBuff","scope":"global","filter":{"category":["键盘乐器","弦乐器","管乐器","打击乐器"]},"cap":2,"excludeSource":true,"directions":[],"excludeAdjacent":false,"valueMode":"absolute"}</x:v>
       </x:c>
       <x:c r="Y61" s="46" t="str">
-        <x:v>使背包中的乐器标签道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
+        <x:v>使背包中的乐器道具各增加[4／5／6／8／10]表演值，最多2件</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6592,7 +6592,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a478579b2a0494e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R047990ab07e8443c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>